<commit_message>
Pasada amplia: EngageTT +4 fuentes (sigue DUDA lean NO); recompilado
3ª pasada amplia refuerza NO en TT (Oxford Insights + MPAAI: IA = chatbot ANANSI +
encuestas, sin Sensemaking sobre aportes); cabo suelto no verificable (403).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/planilla_detalle_casos_ILIA2026.xlsx
+++ b/data/gates/planilla_detalle_casos_ILIA2026.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Evidencia (verbatim)'!$A$1:$L$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'GAPS (buscar manual)'!$A$1:$F$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Fuentes'!$A$1:$F$234</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alertas'!$A$1:$D$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alertas'!$A$1:$D$199</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -13014,7 +13014,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>UNICO CABO ABIERTO tras 2a pasada: el documento 'NDTS 2025 - Actionable Feedback &amp; Implementation Plan' (que sintetiza la retroalimentacion) no pudo recuperarse para verificar si la sintesis/agrupacion del CONTENIDO se hizo con IA (Go Vocal Sensemaking) o manualmente. engage.gov.tt esta bloqueado a nivel de gateway del proxy (HTTP 403 policy denial para engage.gov.tt:443) y ningun buscador expone su texto metodologico. Es lo unico que podria voltear la decision de NO a SI; revisar manualmente.</t>
+          <t>UNICO CABO ABIERTO tras 2a y 3a pasada: el documento 'NDTS 2025 - Actionable Feedback &amp; Implementation Plan' (que sintetiza la retroalimentacion) no pudo recuperarse para verificar si la sintesis/agrupacion del CONTENIDO se hizo con IA (Go Vocal Sensemaking) o manualmente. engage.gov.tt esta bloqueado a nivel de gateway del proxy (HTTP 403 policy denial para engage.gov.tt:443) y ningun buscador expone su texto metodologico; ni siquiera con busqueda AMPLIA en 3a pasada aparece el texto. Es lo unico que podria voltear la decision de NO a SI; revisar manualmente el PDF: https://engage.gov.tt/uploads/51c7a0a3-20e6-46aa-8b13-72bd21a4f9c2/idea_file/file/ac51ce34-6291-4c02-a83f-caa33d60915b/National_Digital_Transformation_Strategy__NDTS__2025_-Actionable_Feedback___Implementation_Plan.pdf</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -21458,7 +21458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D197"/>
+  <dimension ref="A1:D199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -22365,7 +22365,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>[2ª pasada DUDA→DUDA(lean NO)] Tras investigación dirigida (8 búsquedas + 3 fetches, jun-2026) NO se halló evidencia de que ISIDataInsights se haya aplicado a un proceso participativo concreto procesando el CONTENIDO de aportes ciudadanos reales. Toda la documentación (oct-dic 2024) la sitúa en fase PROSPECTIVA ('entra en una tercera etapa, donde será integrada a los sistemas del Distrito' / 'la solución se implementará para que se incorpore a los sistemas'); ninguna fuente de 2025-2026 reporta integración finalizada, despliegue operativo, ni análisis de aportes de un proceso participativo (PDD 2024-2028, POT, consulta, presupuesto participativo). Entretanto la estrategia '5 en Innovación' de la SDP avanzó a retos posteriores (Reto 3 'Ciudad aeroportuaria', GovTech 2025) sin reaparición de la herramienta en uso. Razón de la inclinación a NO: criterio de inclusión exige APLICACIÓN real sobre aportes; aquí solo hay función prevista. Se conserva DUDA(lean NO) porque la evidencia es negativa (ausencia de reportes), no prueba positiva de no-uso.</t>
+          <t>[3ª pasada amplia→DUDA(lean NO)] Búsqueda MÁS AMPLIA (jul-2026, 12+ búsquedas/fetches ES/EN por canales diversos más allá de la SDP: empresa desarrolladora IGG en web/LinkedIn/directorios, dominio del producto, SECOP/datos.gov.co/contratos.gov.co, despliegues en LATAM, y vínculo con procesos participativos concretos PDD/POT/presupuesto) NO logró CERRAR el caso: sigue SIN evidencia de aplicación operativa sobre el CONTENIDO de aportes ciudadanos reales. Nuevos hallazgos que refuerzan NO: (1) ISIDataInsights NO es un producto comercial de IGG con clientes/despliegues (no existe dominio propio ni caso de estudio; solo aparece ligada al reto de la SDP); (2) el único rastro público de IGG con la herramienta es su post de LinkedIn '¡Ganamos!' (~dic 2024) sobre GANAR el concurso, sin publicación posterior de despliegue/resultados; (3) no se halló contrato en SECOP/datos.gov.co que vincule a IGG con la SDP para implementación; (4) sin despliegues en otras ciudades de LATAM; (5) el texto de Maloka/SDP sobre 'metodologías ágiles / sesiones de prueba y validación / capacidades instaladas' describe el DESARROLLO de la herramienta durante la fase del reto, no el análisis de aportes reales (lenguaje de impacto en futuro: 'contribuirá', 'será integrada'); (6) las iniciativas de IA+participación en Bogotá que sí existen (POT con ~20 mil aportes; estudio académico de FACTIBILIDAD de IA para el POT en revista Control Visible; Ecosistema de IA Urbana de $20 mil millones de la Agencia Atenea; agente Chatico) son SEPARADAS y ninguna usa ISIDataInsights sobre aportes. Se mantiene DUDA(lean NO): la evidencia es negativa (ausencia de reportes de uso), no prueba positiva de no-uso; falta un reporte de despliegue de la fase 3 aplicado a aportes de un proceso participativo concreto.</t>
         </is>
       </c>
     </row>
@@ -22387,7 +22387,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>RIESGO DE CONFUSIÓN: existe una iniciativa SEPARADA de la SDP de Bogotá titulada 'Por primera vez la ciudadanía podrá participar en la construcción del Plan de Desarrollo de Bogotá a través de Inteligencia Artificial', que corresponde al agente virtual 'Chatico' (chatbot en WhatsApp para recoger propuestas ciudadanas al PDD 'Bogotá Camina Segura' 2024-2028, con módulo de gobierno abierto). Chatico NO es ISIDataInsights; son sistemas y casos distintos. En la 2ª pasada se confirmó que las fuentes de 2025-2026 sobre IA + participación en planeación de Bogotá refieren Chatico y estudios de factibilidad de IA para el POT, NO ISIDataInsights en uso. Este caso (CO-isidatainsights...) se refiere exclusivamente a la herramienta ganadora del Reto 'Datos con Historia'. No conflar ambos.</t>
+          <t>[2ª pasada DUDA→DUDA(lean NO)] Tras investigación dirigida (8 búsquedas + 3 fetches, jun-2026) NO se halló evidencia de que ISIDataInsights se haya aplicado a un proceso participativo concreto procesando el CONTENIDO de aportes ciudadanos reales. Toda la documentación (oct-dic 2024) la sitúa en fase PROSPECTIVA ('entra en una tercera etapa, donde será integrada a los sistemas del Distrito' / 'la solución se implementará para que se incorpore a los sistemas'); ninguna fuente de 2025-2026 reporta integración finalizada, despliegue operativo, ni análisis de aportes de un proceso participativo (PDD 2024-2028, POT, consulta, presupuesto participativo). Entretanto la estrategia '5 en Innovación' de la SDP avanzó a retos posteriores (Reto 3 'Ciudad aeroportuaria', GovTech 2025) sin reaparición de la herramienta en uso. Razón de la inclinación a NO: criterio de inclusión exige APLICACIÓN real sobre aportes; aquí solo hay función prevista. Se conserva DUDA(lean NO) porque la evidencia es negativa (ausencia de reportes), no prueba positiva de no-uso.</t>
         </is>
       </c>
     </row>
@@ -22409,7 +22409,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Los dominios de las fuentes primarias (sdp.gov.co, maloka.org, eltiempo.com, igg.com.co, secretariageneral.gov.co) devuelven 403 tanto a WebFetch como a curl por policy denial del gateway de egreso. El contenido fue recuperado mediante la herramienta WebSearch (que sí accede al texto subyacente y devuelve fragmentos consistentes y corroborados entre SDP, Maloka y El Tiempo). En consecuencia, las citas en evidencia_verbatim y fuentes reflejan la redacción reportada por el crawler de búsqueda; no fue posible abrir el HTML directo para verificar puntuación/ortografía carácter a carácter, por lo que algunas citas pueden tener variaciones menores respecto al original.</t>
+          <t>RIESGO DE CONFUSIÓN: existe una iniciativa SEPARADA de la SDP de Bogotá titulada 'Por primera vez la ciudadanía podrá participar en la construcción del Plan de Desarrollo de Bogotá a través de Inteligencia Artificial', que corresponde al agente virtual 'Chatico' (chatbot en WhatsApp para recoger propuestas ciudadanas al PDD 'Bogotá Camina Segura' 2024-2028, con módulo de gobierno abierto). Chatico NO es ISIDataInsights; son sistemas y casos distintos. En la 2ª pasada se confirmó que las fuentes de 2025-2026 sobre IA + participación en planeación de Bogotá refieren Chatico y estudios de factibilidad de IA para el POT, NO ISIDataInsights en uso. Este caso (CO-isidatainsights...) se refiere exclusivamente a la herramienta ganadora del Reto 'Datos con Historia'. No conflar ambos.</t>
         </is>
       </c>
     </row>
@@ -22431,29 +22431,29 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>El caso está fuertemente fundamentado para el periodo del concurso (oct-dic 2024) pero carece por completo de evidencia de actividad o despliegue operativo en 2025-2026; la clasificación como 'en desarrollo / implementación' y nivel '1 anuncio' refleja esa ausencia.</t>
+          <t>Los dominios de las fuentes primarias (sdp.gov.co, maloka.org, eltiempo.com, igg.com.co, secretariageneral.gov.co) devuelven 403 tanto a WebFetch como a curl por policy denial del gateway de egreso. El contenido fue recuperado mediante la herramienta WebSearch (que sí accede al texto subyacente y devuelve fragmentos consistentes y corroborados entre SDP, Maloka y El Tiempo). En consecuencia, las citas en evidencia_verbatim y fuentes reflejan la redacción reportada por el crawler de búsqueda; no fue posible abrir el HTML directo para verificar puntuación/ortografía carácter a carácter, por lo que algunas citas pueden tener variaciones menores respecto al original.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MX-guanajuato-inteligente-2024-2030</t>
+          <t>CO-isidatainsights-reto-de-ciudad-datos-con</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
+          <t>ISIDataInsights / Reto de Ciudad 'Datos con Historia' (SDP Bogotá)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_CONVOCANTE: el convocante es el Gobierno del Estado de Guanajuato (entidad subnacional / nivel estatal en el federalismo mexicano), NO un municipio. Por instrucción del índice se clasifica como 'gobierno local' (subnacional) a falta de categoría 'gobierno estatal'; podría argumentarse 'otra institución pública'. Decisión: 'gobierno local'.</t>
+          <t>El caso está fuertemente fundamentado para el periodo del concurso (oct-dic 2024) pero carece por completo de evidencia de actividad o despliegue operativo en 2025-2026; la clasificación como 'en desarrollo / implementación' y nivel '1 anuncio' refleja esa ausencia.</t>
         </is>
       </c>
     </row>
@@ -22475,7 +22475,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_SOFTWARE: no se identificó el software/técnica concreto de IA usado para analizar los aportes (gap central de la investigación). Se confirma el USO de IA sobre el contenido de los aportes, pero no la herramienta específica.</t>
+          <t>ALERTA_CONVOCANTE: el convocante es el Gobierno del Estado de Guanajuato (entidad subnacional / nivel estatal en el federalismo mexicano), NO un municipio. Por instrucción del índice se clasifica como 'gobierno local' (subnacional) a falta de categoría 'gobierno estatal'; podría argumentarse 'otra institución pública'. Decisión: 'gobierno local'.</t>
         </is>
       </c>
     </row>
@@ -22497,7 +22497,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_DOBLE_USO_IA: hay dos usos de IA distintos — (1) análisis/sistematización de aportes ciudadanos para construir el programa (este es el que da elegibilidad, rol_IA=contenido); (2) asistente virtual 'Esperanza' para consultar el programa publicado (rol de atención/consulta, NO el motivo de elegibilidad). No confundirlos.</t>
+          <t>ALERTA_SOFTWARE: no se identificó el software/técnica concreto de IA usado para analizar los aportes (gap central de la investigación). Se confirma el USO de IA sobre el contenido de los aportes, pero no la herramienta específica.</t>
         </is>
       </c>
     </row>
@@ -22519,7 +22519,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_FUENTES_403: todas las URLs .gob.mx, guanajuatointeligente.com y varias de prensa .mx devolvieron HTTP 403 a WebFetch; las citas se recuperaron mediante WebSearch (que sí indexa y devuelve el contenido de esas mismas URLs). Verbatim de metodología sostenido principalmente por la página oficial 'cómo hicimos el programa' vía WebSearch.</t>
+          <t>ALERTA_DOBLE_USO_IA: hay dos usos de IA distintos — (1) análisis/sistematización de aportes ciudadanos para construir el programa (este es el que da elegibilidad, rol_IA=contenido); (2) asistente virtual 'Esperanza' para consultar el programa publicado (rol de atención/consulta, NO el motivo de elegibilidad). No confundirlos.</t>
         </is>
       </c>
     </row>
@@ -22541,7 +22541,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_CONFIANZA: cita clave sobre el análisis de contenido proviene de una sola fuente oficial (página de metodología); la prensa corrobora el uso de IA y la participación de 26k ciudadanos pero tiende a enfatizar la IA aplicada a políticas/consulta ('Esperanza') más que el análisis de aportes. Por eso confianza=MEDIA y no ALTA.</t>
+          <t>ALERTA_FUENTES_403: todas las URLs .gob.mx, guanajuatointeligente.com y varias de prensa .mx devolvieron HTTP 403 a WebFetch; las citas se recuperaron mediante WebSearch (que sí indexa y devuelve el contenido de esas mismas URLs). Verbatim de metodología sostenido principalmente por la página oficial 'cómo hicimos el programa' vía WebSearch.</t>
         </is>
       </c>
     </row>
@@ -22563,7 +22563,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_NIVEL: nivel_consolidacion=2 (uso puntual: la IA se usó una vez para elaborar el programa 2024-2030); no es recurrente (no hay ≥2 ediciones del proceso de elaboración). La plataforma/sitio permanece activa pero el ejercicio participativo con IA fue único.</t>
+          <t>ALERTA_CONFIANZA: cita clave sobre el análisis de contenido proviene de una sola fuente oficial (página de metodología); la prensa corrobora el uso de IA y la participación de 26k ciudadanos pero tiende a enfatizar la IA aplicada a políticas/consulta ('Esperanza') más que el análisis de aportes. Por eso confianza=MEDIA y no ALTA.</t>
         </is>
       </c>
     </row>
@@ -22585,29 +22585,29 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_TRADUCCION_POLITICA: podría argumentarse 'Traducción Política' como etapa adicional, dado que los aportes analizados por IA se transformaron en ejes/estrategias del programa; se mantuvo solo 'Análisis' por ser lo explícitamente sustentado en la cita ('transformar el diálogo social en datos para la toma de decisiones').</t>
+          <t>ALERTA_NIVEL: nivel_consolidacion=2 (uso puntual: la IA se usó una vez para elaborar el programa 2024-2030); no es recurrente (no hay ≥2 ediciones del proceso de elaboración). La plataforma/sitio permanece activa pero el ejercicio participativo con IA fue único.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>PA-mansa-idea-pacto-del-bicentenario</t>
+          <t>MX-guanajuato-inteligente-2024-2030</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
+          <t>Guanajuato InteliGENTE 2024-2030 (Programa de Gobierno del Estado de Guanajuato)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>TEMPORALIDAD (aclaración solicitada): el PROCESO participativo de origen (Pacto del Bicentenario 'Cerrando Brechas' / Panamá Propone) fue 2020-2021 (lanzado nov-2020 por Cortizo; fase de propuestas cerrada feb-2021 con 186.182 propuestas / 212.573 participantes; 172.922 clasificadas en 12 temas). La capa de IA (Mansa Idea) es un tratamiento PUNTUAL de ese corpus histórico, lanzada el 1-abr-2024 para la campaña electoral 2024. ano_inicio se fija en 2024 (año en que se despliega la IA), no en 2020. El proceso participativo subyacente NO está activo; la plataforma con IA sí está/estuvo en línea.</t>
+          <t>ALERTA_TRADUCCION_POLITICA: podría argumentarse 'Traducción Política' como etapa adicional, dado que los aportes analizados por IA se transformaron en ejes/estrategias del programa; se mantuvo solo 'Análisis' por ser lo explícitamente sustentado en la cita ('transformar el diálogo social en datos para la toma de decisiones').</t>
         </is>
       </c>
     </row>
@@ -22629,7 +22629,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>CONVOCANTE (duda resuelta): doble atribución registrada. Gobierno nacional convoca el proceso participativo (recolección); sociedad civil (Fundación Panamá Participa) desarrolla y opera la IA. tipo_organizacion='Privado' por el agente que aplica la IA; tipo_desarrollador_IA=['Sociedad Civil'], origen 'Nacional' (Panamá).</t>
+          <t>TEMPORALIDAD (aclaración solicitada): el PROCESO participativo de origen (Pacto del Bicentenario 'Cerrando Brechas' / Panamá Propone) fue 2020-2021 (lanzado nov-2020 por Cortizo; fase de propuestas cerrada feb-2021 con 186.182 propuestas / 212.573 participantes; 172.922 clasificadas en 12 temas). La capa de IA (Mansa Idea) es un tratamiento PUNTUAL de ese corpus histórico, lanzada el 1-abr-2024 para la campaña electoral 2024. ano_inicio se fija en 2024 (año en que se despliega la IA), no en 2020. El proceso participativo subyacente NO está activo; la plataforma con IA sí está/estuvo en línea.</t>
         </is>
       </c>
     </row>
@@ -22651,7 +22651,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>TECNOLOGÍA DE IA NO IDENTIFICADA (duda central abierta): ninguna fuente pública hallada detalla el método técnico de IA de Mansa Idea (clustering/NLP/embeddings/búsqueda semántica/LLM). Se confirma POR DESCRIPCIÓN que la IA actúa sobre el CONTENIDO de los aportes (agrega/organiza/hace navegables 175.000+ propuestas y recoge consensos nacionales y provinciales), suficiente para rol_IA='contenido' y entra_tentativo=SI, pero tipos_IA_familia=[] y usa_LLM_generativa='no-claro' por falta de detalle. El sitio oficial mansaidea.com devuelve 403 a WebFetch.</t>
+          <t>CONVOCANTE (duda resuelta): doble atribución registrada. Gobierno nacional convoca el proceso participativo (recolección); sociedad civil (Fundación Panamá Participa) desarrolla y opera la IA. tipo_organizacion='Privado' por el agente que aplica la IA; tipo_desarrollador_IA=['Sociedad Civil'], origen 'Nacional' (Panamá).</t>
         </is>
       </c>
     </row>
@@ -22673,7 +22673,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>FUENTES: el sitio oficial (mansaidea.com) y los medios panameños (panama24horas.com.pa, laestrella.com.pa) y PNUD devuelven HTTP 403 a WebFetch; el contenido y las citas se recuperaron de forma convergente y consistente mediante WebSearch (múltiples consultas sobre las mismas URLs). Las citas verbatim son reconstrucciones del texto devuelto por WebSearch, no transcripción directa de la página renderizada. Aun así, la convergencia de ≥2 fuentes independientes de prensa + datos oficiales del PNUD sobre el Pacto sustenta confianza ALTA en los hechos centrales (qué es, quién, cuándo, qué hace la IA).</t>
+          <t>TECNOLOGÍA DE IA NO IDENTIFICADA (duda central abierta): ninguna fuente pública hallada detalla el método técnico de IA de Mansa Idea (clustering/NLP/embeddings/búsqueda semántica/LLM). Se confirma POR DESCRIPCIÓN que la IA actúa sobre el CONTENIDO de los aportes (agrega/organiza/hace navegables 175.000+ propuestas y recoge consensos nacionales y provinciales), suficiente para rol_IA='contenido' y entra_tentativo=SI, pero tipos_IA_familia=[] y usa_LLM_generativa='no-claro' por falta de detalle. El sitio oficial mansaidea.com devuelve 403 a WebFetch.</t>
         </is>
       </c>
     </row>
@@ -22695,7 +22695,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>CIFRA DE PROPUESTAS: las fuentes oscilan entre '170.000' y 'más de 175.000' propuestas en Mansa Idea; el dato oficial del Pacto registra 186.182 propuestas recibidas y 172.922 clasificadas tras filtro técnico. La discrepancia se debe a si se cuenta el total recibido, el clasificado o el publicado en la plataforma.</t>
+          <t>FUENTES: el sitio oficial (mansaidea.com) y los medios panameños (panama24horas.com.pa, laestrella.com.pa) y PNUD devuelven HTTP 403 a WebFetch; el contenido y las citas se recuperaron de forma convergente y consistente mediante WebSearch (múltiples consultas sobre las mismas URLs). Las citas verbatim son reconstrucciones del texto devuelto por WebSearch, no transcripción directa de la página renderizada. Aun así, la convergencia de ≥2 fuentes independientes de prensa + datos oficiales del PNUD sobre el Pacto sustenta confianza ALTA en los hechos centrales (qué es, quién, cuándo, qué hace la IA).</t>
         </is>
       </c>
     </row>
@@ -22717,29 +22717,29 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>NOMBRE: el título exacto del proceso es 'Pacto del Bicentenario, Cerrando Brechas' (gerundio); el caso_id usa 'Cerremos la Brecha'. Es la misma iniciativa; se conserva el nombre_caso del encargo.</t>
+          <t>CIFRA DE PROPUESTAS: las fuentes oscilan entre '170.000' y 'más de 175.000' propuestas en Mansa Idea; el dato oficial del Pacto registra 186.182 propuestas recibidas y 172.922 clasificadas tras filtro técnico. La discrepancia se debe a si se cuenta el total recibido, el clasificado o el publicado en la plataforma.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>BR-catedra-brasil-co-lab-usp-ia-generativa</t>
+          <t>PA-mansa-idea-pacto-del-bicentenario</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Cátedra Brasil / Co:Lab USP - IA generativa en presupuesto participativo (SP)</t>
+          <t>Mansa Idea (Pacto del Bicentenario "Cerremos la Brecha", Panamá)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>ESTADO = INVESTIGACIÓN / PROTOTIPO en curso ('Pesquisas em Andamento'), NO despliegue oficial confirmado. El orçamento participativo de São Paulo opera vía Participe+/Participe Mais sin IA generativa verificada en producción.</t>
+          <t>NOMBRE: el título exacto del proceso es 'Pacto del Bicentenario, Cerrando Brechas' (gerundio); el caso_id usa 'Cerremos la Brecha'. Es la misma iniciativa; se conserva el nombre_caso del encargo.</t>
         </is>
       </c>
     </row>
@@ -22761,7 +22761,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Convocante/desarrollador = universidad (USP / EACH / Co:Lab / GETIP), no gobierno; reduce elegibilidad como caso de proceso participativo con IA desplegada.</t>
+          <t>ESTADO = INVESTIGACIÓN / PROTOTIPO en curso ('Pesquisas em Andamento'), NO despliegue oficial confirmado. El orçamento participativo de São Paulo opera vía Participe+/Participe Mais sin IA generativa verificada en producción.</t>
         </is>
       </c>
     </row>
@@ -22783,7 +22783,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Limitación de evidencia: las 3 fuentes primarias (blog Co:Lab, Jornal da USP, Policy Brief PDF) devolvieron HTTP 403 vía WebFetch (bloqueo del proxy); las citas se obtuvieron de snippets de búsqueda y no son citas textuales completas verificadas del cuerpo. Confianza limitada a MEDIA.</t>
+          <t>Convocante/desarrollador = universidad (USP / EACH / Co:Lab / GETIP), no gobierno; reduce elegibilidad como caso de proceso participativo con IA desplegada.</t>
         </is>
       </c>
     </row>
@@ -22805,14 +22805,14 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>El ejemplo concreto (IA ayuda a redactar propuesta de 'rede de ciclovias na zona leste') describe el rol de la IA sobre el CONTENIDO del aporte; si en el futuro se confirma despliegue real en el proceso participativo, el caso podría reclasificarse a entra=SI.</t>
+          <t>Limitación de evidencia: las 3 fuentes primarias (blog Co:Lab, Jornal da USP, Policy Brief PDF) devolvieron HTTP 403 vía WebFetch (bloqueo del proxy); las citas se obtuvieron de snippets de búsqueda y no son citas textuales completas verificadas del cuerpo. Confianza limitada a MEDIA.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>BR-opa-piaui-presupuesto-participativo-digi</t>
+          <t>BR-catedra-brasil-co-lab-usp-ia-generativa</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -22822,12 +22822,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>OPA Piauí - Orçamento Participativo Digital (Colab + AWS)</t>
+          <t>Cátedra Brasil / Co:Lab USP - IA generativa en presupuesto participativo (SP)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>[2ª pasada DUDA→NO] La pregunta binaria se resuelve en CONTRA del análisis de contenido: en el OPA la IA solo se documenta como aceleración del 'processamento' (-40% tempo) + seguridad (filtrar conexões inseguras vía AWS CloudFront) + chatbot/capacitación (CapacitIA) + panel de transparencia (Observatório do OPA). La 'análise técnica' de viabilidad la hacen reiteradamente 'equipes técnicas' (humanas). La AWS citada es cómputo/BD/seguridad (EC2, RDS, CloudFront), no ML de contenido. La única atribución de IA que 'agrupa ideias por eixo temático' corresponde a OTRO proceso (Diálogos pelo Piauí / PPA), no al OPA, y ni siquiera se confirmó verbatim. Bajo el criterio del índice (solo processamento/triaje + infraestructura/seguridad → NO; rol_IA='apoyo'), NO ENTRA. Incertidumbre residual NO decisiva: falta documentación técnica primaria de Colab Gov.AI específica del OPA (gov.br y colab.com.br dan 403).</t>
+          <t>El ejemplo concreto (IA ayuda a redactar propuesta de 'rede de ciclovias na zona leste') describe el rol de la IA sobre el CONTENIDO del aporte; si en el futuro se confirma despliegue real en el proceso participativo, el caso podría reclasificarse a entra=SI.</t>
         </is>
       </c>
     </row>
@@ -22849,7 +22849,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>PROCESOS DISTINTOS (no confundir): (a) OPA = Orçamento Participativo Digital (presupuesto participativo, propuestas de entidades + votación popular); (b) 'Diálogos pelo Piauí' = escucha popular para revisión del PPA 2024-2027 (oficinas presenciales en 12 Territórios). La señal de IA que 'agrupa ideias semelhantes' / 'estrutura propostas por eixo' apareció ligada a (b), NO a (a). Esta ficha es de (a) OPA.</t>
+          <t>[2ª pasada DUDA→NO] La pregunta binaria se resuelve en CONTRA del análisis de contenido: en el OPA la IA solo se documenta como aceleración del 'processamento' (-40% tempo) + seguridad (filtrar conexões inseguras vía AWS CloudFront) + chatbot/capacitación (CapacitIA) + panel de transparencia (Observatório do OPA). La 'análise técnica' de viabilidad la hacen reiteradamente 'equipes técnicas' (humanas). La AWS citada es cómputo/BD/seguridad (EC2, RDS, CloudFront), no ML de contenido. La única atribución de IA que 'agrupa ideias por eixo temático' corresponde a OTRO proceso (Diálogos pelo Piauí / PPA), no al OPA, y ni siquiera se confirmó verbatim. Bajo el criterio del índice (solo processamento/triaje + infraestructura/seguridad → NO; rol_IA='apoyo'), NO ENTRA. Incertidumbre residual NO decisiva: falta documentación técnica primaria de Colab Gov.AI específica del OPA (gov.br y colab.com.br dan 403).</t>
         </is>
       </c>
     </row>
@@ -22871,7 +22871,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>FUENTES: todas las URLs gov.br (pi.gov.br, portal.pi.gov.br, seplan.pi.gov.br, sia.pi.gov.br, opa.seplan.pi.gov.br) y colab.com.br devuelven HTTP 403 a WebFetch; el contenido y las citas se recuperaron de forma convergente mediante WebSearch (múltiples consultas en PT/ES/EN). Las citas verbatim son texto devuelto por WebSearch sobre esas URLs, no transcripción directa de la página renderizada; por ello confianza MEDIA.</t>
+          <t>PROCESOS DISTINTOS (no confundir): (a) OPA = Orçamento Participativo Digital (presupuesto participativo, propuestas de entidades + votación popular); (b) 'Diálogos pelo Piauí' = escucha popular para revisión del PPA 2024-2027 (oficinas presenciales en 12 Territórios). La señal de IA que 'agrupa ideias semelhantes' / 'estrutura propostas por eixo' apareció ligada a (b), NO a (a). Esta ficha es de (a) OPA.</t>
         </is>
       </c>
     </row>
@@ -22893,7 +22893,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>DESARROLLADOR: la capacidad de IA está en la plataforma Colab Gov / Colab Gov.AI (govtech Colab, empresa brasileña = Privado) sobre infraestructura AWS (Amazon, Privado/Internacional). tipo_desarrollador_IA=['Privado'], origen_desarrollador='Internacional' por el peso de AWS; podría matizarse a 'Nacional' si la IA fuese desarrollo propio de Colab.</t>
+          <t>FUENTES: todas las URLs gov.br (pi.gov.br, portal.pi.gov.br, seplan.pi.gov.br, sia.pi.gov.br, opa.seplan.pi.gov.br) y colab.com.br devuelven HTTP 403 a WebFetch; el contenido y las citas se recuperaron de forma convergente mediante WebSearch (múltiples consultas en PT/ES/EN). Las citas verbatim son texto devuelto por WebSearch sobre esas URLs, no transcripción directa de la página renderizada; por ello confianza MEDIA.</t>
         </is>
       </c>
     </row>
@@ -22915,7 +22915,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>CONVOCANTE: Gobierno del ESTADO de Piauí (nivel subnacional). Por convención del índice se clasifica 'gobierno local' (no nacional). Coordina SEPLAN; apoya Seres; existe además una Secretaria de Inteligência Artificial (SIA) estatal vinculada a la capacitación (CapacitIA) del OPA.</t>
+          <t>DESARROLLADOR: la capacidad de IA está en la plataforma Colab Gov / Colab Gov.AI (govtech Colab, empresa brasileña = Privado) sobre infraestructura AWS (Amazon, Privado/Internacional). tipo_desarrollador_IA=['Privado'], origen_desarrollador='Internacional' por el peso de AWS; podría matizarse a 'Nacional' si la IA fuese desarrollo propio de Colab.</t>
         </is>
       </c>
     </row>
@@ -22937,7 +22937,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>CONSOLIDACIÓN: nivel 3 (recurrente, ≥2 ediciones) confirmado: ediciones OPA 2023-2024, 2024-2025, 2025-2026 y 2026-2027 (cuatro ciclos), con votación récord creciente (273.890 votos válidos en 2025-2026; &gt;300 mil participaciones en la votación). continuidad='Plataforma' (Colab Gov es plataforma permanente del proceso).</t>
+          <t>CONVOCANTE: Gobierno del ESTADO de Piauí (nivel subnacional). Por convención del índice se clasifica 'gobierno local' (no nacional). Coordina SEPLAN; apoya Seres; existe además una Secretaria de Inteligência Artificial (SIA) estatal vinculada a la capacitación (CapacitIA) del OPA.</t>
         </is>
       </c>
     </row>
@@ -22959,29 +22959,29 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>CONTEXTO IA en Piauí: Piauí es el único estado de Brasil con una Secretaría de Inteligencia Artificial (SIA) y desarrolla un proyecto de LLM en portugués. Esto refuerza la plausibilidad de uso de IA, pero NO constituye evidencia de que un LLM/IA se aplique al análisis de CONTENIDO de las propuestas del OPA; los usos confirmados de la SIA en el OPA son capacitación (CapacitIA), un chatbot de atención y un panel de transparencia.</t>
+          <t>CONSOLIDACIÓN: nivel 3 (recurrente, ≥2 ediciones) confirmado: ediciones OPA 2023-2024, 2024-2025, 2025-2026 y 2026-2027 (cuatro ciclos), con votación récord creciente (273.890 votos válidos en 2025-2026; &gt;300 mil participaciones en la votación). continuidad='Plataforma' (Colab Gov es plataforma permanente del proceso).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>CL-senador-virtual-crowdlaw-goblab-uai-imfd</t>
+          <t>BR-opa-piaui-presupuesto-participativo-digi</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Senador Virtual / CrowdLaw (GobLab UAI + IMFD)</t>
+          <t>OPA Piauí - Orçamento Participativo Digital (Colab + AWS)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>[2a pasada DUDA-&gt;NO] El componente con IA/NLP (GobLab UAI + Harvard, proyecto CrowdLaw) es INVESTIGACION ACADEMICA cuyo producto son RECOMENDACIONES, no un despliegue. La fuente decisiva es '16 years of CrowdLaw': para aprovechar la plataforma hay que 'add a reliable methodology for processing citizen input' (algo aun NO implementado), y Guridi et al. (Cornell, arXiv 2410.22937, 2024) concluyen que los gobiernos 'are not widely adopting' NLP para analizar las contribuciones ciudadanas. No se hallo ninguna evidencia 2024-2026 de un sistema de NLP en produccion integrado al proceso del Senado que sistematice los aportes de Senador Virtual. Por tanto entra_tentativo=NO, usa_IA_en_proceso=no, confianza=ALTA.</t>
+          <t>CONTEXTO IA en Piauí: Piauí es el único estado de Brasil con una Secretaría de Inteligencia Artificial (SIA) y desarrolla un proyecto de LLM en portugués. Esto refuerza la plausibilidad de uso de IA, pero NO constituye evidencia de que un LLM/IA se aplique al análisis de CONTENIDO de las propuestas del OPA; los usos confirmados de la SIA en el OPA son capacitación (CapacitIA), un chatbot de atención y un panel de transparencia.</t>
         </is>
       </c>
     </row>
@@ -23003,7 +23003,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>DESAMBIGUACION CLAVE (confirmada): la 'senial IMFD + NLP' del prompt corresponde a la plataforma 'Vincula' del IMFD, que 'applies natural language processing (NLP) techniques... allows linking topics of interest with academics' para conectar academia&lt;-&gt;Congreso; NO procesa los aportes ciudadanos de Senador Virtual. No hay evidencia de que el IMFD aplique NLP al contenido de los aportes de Senador Virtual.</t>
+          <t>[2a pasada DUDA-&gt;NO] El componente con IA/NLP (GobLab UAI + Harvard, proyecto CrowdLaw) es INVESTIGACION ACADEMICA cuyo producto son RECOMENDACIONES, no un despliegue. La fuente decisiva es '16 years of CrowdLaw': para aprovechar la plataforma hay que 'add a reliable methodology for processing citizen input' (algo aun NO implementado), y Guridi et al. (Cornell, arXiv 2410.22937, 2024) concluyen que los gobiernos 'are not widely adopting' NLP para analizar las contribuciones ciudadanas. No se hallo ninguna evidencia 2024-2026 de un sistema de NLP en produccion integrado al proceso del Senado que sistematice los aportes de Senador Virtual. Por tanto entra_tentativo=NO, usa_IA_en_proceso=no, confianza=ALTA.</t>
         </is>
       </c>
     </row>
@@ -23025,7 +23025,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>DESAMBIGUACION (2a pasada): ArChileBot (Camara de Diputadas y Diputados, presentado en el marco del proyecto IDEA Internacional/UE) es un chatbot de BUSQUEDA DOCUMENTAL en lenguaje natural sobre archivos/leyes historicas, inspirado en el ArchiBot del Parlamento Europeo; NO sistematiza los aportes ciudadanos de Senador Virtual. Tampoco aplica 'Parlamento AI' (P. Matamoros), que monitorea DEBATES legislativos, no aportes ciudadanos.</t>
+          <t>DESAMBIGUACION CLAVE (confirmada): la 'senial IMFD + NLP' del prompt corresponde a la plataforma 'Vincula' del IMFD, que 'applies natural language processing (NLP) techniques... allows linking topics of interest with academics' para conectar academia&lt;-&gt;Congreso; NO procesa los aportes ciudadanos de Senador Virtual. No hay evidencia de que el IMFD aplique NLP al contenido de los aportes de Senador Virtual.</t>
         </is>
       </c>
     </row>
@@ -23047,7 +23047,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>La plataforma Senador Virtual / Congreso Virtual en si NO usa IA sobre el contenido de los aportes; la actualizacion BID (2018-2020) anadio 'mejoras tecnologicas para analizar los comentarios registrados y crear un reporte con visualizaciones para la comision' (analitica descriptiva/visualizacion), no NLP/IA generativa confirmados. La plataforma sola no basta para elegibilidad.</t>
+          <t>DESAMBIGUACION (2a pasada): ArChileBot (Camara de Diputadas y Diputados, presentado en el marco del proyecto IDEA Internacional/UE) es un chatbot de BUSQUEDA DOCUMENTAL en lenguaje natural sobre archivos/leyes historicas, inspirado en el ArchiBot del Parlamento Europeo; NO sistematiza los aportes ciudadanos de Senador Virtual. Tampoco aplica 'Parlamento AI' (P. Matamoros), que monitorea DEBATES legislativos, no aportes ciudadanos.</t>
         </is>
       </c>
     </row>
@@ -23069,7 +23069,7 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>nivel_consolidacion=3 y estado_actividad=activo se refieren a la PLATAFORMA participativa (&gt;16 anios, multiples ediciones, &gt;130.000 participantes, activa en 2026), no a un componente de IA. La consolidacion del eventual componente IA seria ~0-1 (investigacion/recomendacion).</t>
+          <t>La plataforma Senador Virtual / Congreso Virtual en si NO usa IA sobre el contenido de los aportes; la actualizacion BID (2018-2020) anadio 'mejoras tecnologicas para analizar los comentarios registrados y crear un reporte con visualizaciones para la comision' (analitica descriptiva/visualizacion), no NLP/IA generativa confirmados. La plataforma sola no basta para elegibilidad.</t>
         </is>
       </c>
     </row>
@@ -23091,7 +23091,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Anti-bot: todas las URLs de UAI (goblab/gobierno/ciudadaniadigital), imfd.cl, arxiv.org (abs y html), medium.com, owlstown.net y github.io del autor devolvieron HTTP 403 a WebFetch (anti-bot del origen, no fallo del proxy). Verbatim reconstruido via WebSearch con extractos convergentes en multiples consultas; senado.cl, congresovirtual.cl, sagepub e idea.int quedan como 'no-verificado' por no haberse fetcheado el HTML.</t>
+          <t>nivel_consolidacion=3 y estado_actividad=activo se refieren a la PLATAFORMA participativa (&gt;16 anios, multiples ediciones, &gt;130.000 participantes, activa en 2026), no a un componente de IA. La consolidacion del eventual componente IA seria ~0-1 (investigacion/recomendacion).</t>
         </is>
       </c>
     </row>
@@ -23113,29 +23113,29 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>ano_inicio=2018 se asigna por el convenio Senado-BID y el arranque de la linea CrowdLaw; la plataforma base (Senador Virtual) existe desde 2003 y el relanzamiento 'Congreso Virtual' es 2020. tipo_desarrollador_IA=Academia y origen=Nacional describen el eventual componente de investigacion (GobLab UAI + Harvard + IMFD); Harvard introduce un origen Internacional en la alianza de investigacion, pero el desarrollador principal es nacional (UAI/IMFD).</t>
+          <t>Anti-bot: todas las URLs de UAI (goblab/gobierno/ciudadaniadigital), imfd.cl, arxiv.org (abs y html), medium.com, owlstown.net y github.io del autor devolvieron HTTP 403 a WebFetch (anti-bot del origen, no fallo del proxy). Verbatim reconstruido via WebSearch con extractos convergentes en multiples consultas; senado.cl, congresovirtual.cl, sagepub e idea.int quedan como 'no-verificado' por no haberse fetcheado el HTML.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>CO-dnp-dialogos-regionales-vinculantes-pnd</t>
+          <t>CL-senador-virtual-crowdlaw-goblab-uai-imfd</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>DNP - Diálogos Regionales Vinculantes (PND 2022-2026)</t>
+          <t>Senador Virtual / CrowdLaw (GobLab UAI + IMFD)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>[2ª pasada DUDA→NO] Investigación dirigida (≈10 búsquedas/fetches, ES/EN) CONFIRMA que la sistematización de las 89.788 propuestas usó lectura + FRECUENCIA/RECURRENCIA + categorización en categorías predefinidas + nubes de palabras/visor, SIN evidencia de NLP/ML/topic modeling/clustering sobre el contenido. Señales decisivas en contra de IA: (1) el GitHub oficial de la Unidad de Científicos de Datos (ucd-dnp, 7 repos) NO tiene proyecto de DRV y su única librería NLP ('ConTexto') no se vincula al ejercicio; (2) búsqueda EN con términos NLP/ML/text-mining → 0 resultados sobre los DRV; (3) críticos (Dejusticia: 'no había funcionarios con computadores sistematizando... propuestas guardadas en notas de voz de celular'; FIP; CCONG: 'el proceso con que se sistematizaron las demandas nunca se identificó con claridad') denuncian la AUSENCIA de método automatizado. Análisis por frecuencia + categorización manual ≠ IA según el criterio del índice → NO entra.</t>
+          <t>ano_inicio=2018 se asigna por el convenio Senado-BID y el arranque de la linea CrowdLaw; la plataforma base (Senador Virtual) existe desde 2003 y el relanzamiento 'Congreso Virtual' es 2020. tipo_desarrollador_IA=Academia y origen=Nacional describen el eventual componente de investigacion (GobLab UAI + Harvard + IMFD); Harvard introduce un origen Internacional en la alianza de investigacion, pero el desarrollador principal es nacional (UAI/IMFD).</t>
         </is>
       </c>
     </row>
@@ -23157,7 +23157,7 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Riesgo de falso positivo descartado: 'Unidad de Científicos de Datos' y 'análisis cuantitativo' sugieren IA, pero todas las fuentes solo respaldan estadística de frecuencia, agrupación en categorías y visualización (nubes de palabras, barras, visor); no asumir NLP sin documento técnico, que no la respalda.</t>
+          <t>[2ª pasada DUDA→NO] Investigación dirigida (≈10 búsquedas/fetches, ES/EN) CONFIRMA que la sistematización de las 89.788 propuestas usó lectura + FRECUENCIA/RECURRENCIA + categorización en categorías predefinidas + nubes de palabras/visor, SIN evidencia de NLP/ML/topic modeling/clustering sobre el contenido. Señales decisivas en contra de IA: (1) el GitHub oficial de la Unidad de Científicos de Datos (ucd-dnp, 7 repos) NO tiene proyecto de DRV y su única librería NLP ('ConTexto') no se vincula al ejercicio; (2) búsqueda EN con términos NLP/ML/text-mining → 0 resultados sobre los DRV; (3) críticos (Dejusticia: 'no había funcionarios con computadores sistematizando... propuestas guardadas en notas de voz de celular'; FIP; CCONG: 'el proceso con que se sistematizaron las demandas nunca se identificó con claridad') denuncian la AUSENCIA de método automatizado. Análisis por frecuencia + categorización manual ≠ IA según el criterio del índice → NO entra.</t>
         </is>
       </c>
     </row>
@@ -23179,7 +23179,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Limitación de acceso (residual): el dominio oficial dnp.gov.co / colaboracion.dnp.gov.co / sispt.dnp.gov.co / funcionpublica.gov.co y varios PDFs académicos devuelven HTTP 403 vía WebFetch; la evidencia verbatim proviene mayormente de snippets de buscador, no de lectura directa de la fuente primaria. La convergencia entre fuentes oficiales, académicas (Externado) y críticas (Dejusticia/FIP/CCONG) es, no obstante, suficiente para resolver en NO con confianza MEDIA.</t>
+          <t>Riesgo de falso positivo descartado: 'Unidad de Científicos de Datos' y 'análisis cuantitativo' sugieren IA, pero todas las fuentes solo respaldan estadística de frecuencia, agrupación en categorías y visualización (nubes de palabras, barras, visor); no asumir NLP sin documento técnico, que no la respalda.</t>
         </is>
       </c>
     </row>
@@ -23201,14 +23201,14 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Existen análisis académicos de terceros con minería de texto sobre datos relacionados (p. ej. arXiv 2504.04325 sobre audiencias de la JEP), pero corresponden a OTRO proceso (JEP), no a los DRV; no usar como evidencia de IA en los DRV.</t>
+          <t>Limitación de acceso (residual): el dominio oficial dnp.gov.co / colaboracion.dnp.gov.co / sispt.dnp.gov.co / funcionpublica.gov.co y varios PDFs académicos devuelven HTTP 403 vía WebFetch; la evidencia verbatim proviene mayormente de snippets de buscador, no de lectura directa de la fuente primaria. La convergencia entre fuentes oficiales, académicas (Externado) y críticas (Dejusticia/FIP/CCONG) es, no obstante, suficiente para resolver en NO con confianza MEDIA.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>CO-ia-para-participacion-en-el-pot-de-bogot</t>
+          <t>CO-dnp-dialogos-regionales-vinculantes-pnd</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -23218,12 +23218,12 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>IA para participación en el POT de Bogotá (Control Visible / Auditoría General)</t>
+          <t>DNP - Diálogos Regionales Vinculantes (PND 2022-2026)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>[2ª pasada DUDA-&gt;NO] Tras investigación dirigida (8 búsquedas web + 4 intentos de fetch), se confirma que el caso es ÚNICAMENTE un ARTÍCULO ACADÉMICO/ESTUDIO EXPLORATORIO (Fundación Universitaria del Área Andina, Maestría en Innovación; revista Control Visible de la Auditoría General) que PROPONE y mide la 'factibilidad de aceptación' de una herramienta de IA para la participación en el POT encuestando a 395 ciudadanos y entrevistando expertos. NO existe despliegue institucional que aplique IA al CONTENIDO de aportes ciudadanos reales del POT. Los despliegues reales de IA de la SDP que aparecen en las búsquedas (ISIDataInsights/'Inteligencia 360°'/reto 'Datos con Historia'; Chatico) están ligados al Plan Distrital de DESARROLLO 'Bogotá Camina Segura' 2024-2028 —NO al POT— y son casos distintos. Por ser propuesta/estudio sin despliegue institucional sobre el POT -&gt; veredicto NO, confianza ALTA.</t>
+          <t>Existen análisis académicos de terceros con minería de texto sobre datos relacionados (p. ej. arXiv 2504.04325 sobre audiencias de la JEP), pero corresponden a OTRO proceso (JEP), no a los DRV; no usar como evidencia de IA en los DRV.</t>
         </is>
       </c>
     </row>
@@ -23245,7 +23245,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>DISTINCIÓN CONVOCANTE vs AUTOR: El convocante del PROCESO participativo de referencia (POT) sería el gobierno local (Secretaría Distrital de Planeación / Concejo de Bogotá), pero el ESTUDIO lo realizan autores académicos (Areandina) y lo publica la Auditoría General como editora de revista. Para tipo_convocante se consigna 'universidad' por ser quien produce/conduce el caso documentado (el estudio); NO se atribuye a la Auditoría la ejecución de la herramienta (solo edita la revista), ni se atribuye al gobierno local un despliegue que no se documenta.</t>
+          <t>[2ª pasada DUDA-&gt;NO] Tras investigación dirigida (8 búsquedas web + 4 intentos de fetch), se confirma que el caso es ÚNICAMENTE un ARTÍCULO ACADÉMICO/ESTUDIO EXPLORATORIO (Fundación Universitaria del Área Andina, Maestría en Innovación; revista Control Visible de la Auditoría General) que PROPONE y mide la 'factibilidad de aceptación' de una herramienta de IA para la participación en el POT encuestando a 395 ciudadanos y entrevistando expertos. NO existe despliegue institucional que aplique IA al CONTENIDO de aportes ciudadanos reales del POT. Los despliegues reales de IA de la SDP que aparecen en las búsquedas (ISIDataInsights/'Inteligencia 360°'/reto 'Datos con Historia'; Chatico) están ligados al Plan Distrital de DESARROLLO 'Bogotá Camina Segura' 2024-2028 —NO al POT— y son casos distintos. Por ser propuesta/estudio sin despliegue institucional sobre el POT -&gt; veredicto NO, confianza ALTA.</t>
         </is>
       </c>
     </row>
@@ -23267,7 +23267,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>ACCESO BLOQUEADO (corregido en 2ª pasada): El dominio controlvisible.auditoria.gov.co (y sdp.gov.co, scholar.google.com) devuelve HTTP 403 Forbidden a WebFetch. A diferencia de lo asumido en la 1ª pasada, el proxy de egreso reporta estado 'healthy' sin fallos de relay (recentRelayFailures vacío), por lo que el 403 es respuesta del SERVIDOR DE ORIGEN (probable anti-bot/WAF), no un policy denial del gateway. Todo el contenido verbatim y los metadatos se recuperaron de forma consistente vía WebSearch en múltiples consultas independientes. No se pudo verificar puntuación/ortografía carácter a carácter ni listar nombres de autores; una cita de tipo_convocante quedó solo en su versión en inglés (paráfrasis de WebSearch) y se marca como tal.</t>
+          <t>DISTINCIÓN CONVOCANTE vs AUTOR: El convocante del PROCESO participativo de referencia (POT) sería el gobierno local (Secretaría Distrital de Planeación / Concejo de Bogotá), pero el ESTUDIO lo realizan autores académicos (Areandina) y lo publica la Auditoría General como editora de revista. Para tipo_convocante se consigna 'universidad' por ser quien produce/conduce el caso documentado (el estudio); NO se atribuye a la Auditoría la ejecución de la herramienta (solo edita la revista), ni se atribuye al gobierno local un despliegue que no se documenta.</t>
         </is>
       </c>
     </row>
@@ -23289,29 +23289,29 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>NO CONFUNDIR con casos distintos hallados en las búsquedas que SÍ son despliegues institucionales y constituyen otros casos potenciales (todos ligados al Plan Distrital de DESARROLLO, no al POT): (a) Secretaría Distrital de Planeación de Bogotá — 'Por primera vez la ciudadanía podrá participar en la construcción del Plan de Desarrollo de Bogotá a través de Inteligencia Artificial' (sdp.gov.co); (b) 'Chatico', asistente virtual de Bogotá (participación en el Plan de Desarrollo vía WhatsApp); (c) ISIDataInsights / 'Inteligencia 360°' / reto 'Datos con Historia' (oct-nov 2024, estrategia '5 en Innovación' del Plan de Desarrollo). Ninguno aplica IA a aportes del POT y no deben fusionarse con esta ficha.</t>
+          <t>ACCESO BLOQUEADO (corregido en 2ª pasada): El dominio controlvisible.auditoria.gov.co (y sdp.gov.co, scholar.google.com) devuelve HTTP 403 Forbidden a WebFetch. A diferencia de lo asumido en la 1ª pasada, el proxy de egreso reporta estado 'healthy' sin fallos de relay (recentRelayFailures vacío), por lo que el 403 es respuesta del SERVIDOR DE ORIGEN (probable anti-bot/WAF), no un policy denial del gateway. Todo el contenido verbatim y los metadatos se recuperaron de forma consistente vía WebSearch en múltiples consultas independientes. No se pudo verificar puntuación/ortografía carácter a carácter ni listar nombres de autores; una cita de tipo_convocante quedó solo en su versión en inglés (paráfrasis de WebSearch) y se marca como tal.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>CU-consulta-popular-codigo-de-las-familias</t>
+          <t>CO-ia-para-participacion-en-el-pot-de-bogot</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>CU</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Consulta Popular Código de las Familias (GEMA-CEN / XISCOP)</t>
+          <t>IA para participación en el POT de Bogotá (Control Visible / Auditoría General)</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Caso clasificado en bloque '1-dudoso'. DUDA CENTRAL (¿IA real vs lógica de reglas?) RESUELTA hacia SI: la ficha técnica oficial de GEMA (Datys) lo describe como herramienta de análisis de grandes volúmenes de archivos con recuperación de información, clasificación por temáticas, OCR, agrupamiento de documentos similares y resumen automático extractivo -&gt; NLP/minería de texto/recuperación de información sobre el CONTENIDO, no mero conteo ni agrupación determinista trivial.</t>
+          <t>NO CONFUNDIR con casos distintos hallados en las búsquedas que SÍ son despliegues institucionales y constituyen otros casos potenciales (todos ligados al Plan Distrital de DESARROLLO, no al POT): (a) Secretaría Distrital de Planeación de Bogotá — 'Por primera vez la ciudadanía podrá participar en la construcción del Plan de Desarrollo de Bogotá a través de Inteligencia Artificial' (sdp.gov.co); (b) 'Chatico', asistente virtual de Bogotá (participación en el Plan de Desarrollo vía WhatsApp); (c) ISIDataInsights / 'Inteligencia 360°' / reto 'Datos con Historia' (oct-nov 2024, estrategia '5 en Innovación' del Plan de Desarrollo). Ninguno aplica IA a aportes del POT y no deben fusionarse con esta ficha.</t>
         </is>
       </c>
     </row>
@@ -23333,7 +23333,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Persiste incertidumbre sobre la PROFUNDIDAD técnica del agrupamiento: las fuentes no confirman si usa ML/embeddings semánticos o similitud clásica de recuperación de información. En ambos escenarios se trata de procesamiento de texto sobre el contenido de los aportes, por lo que rol_IA=contenido y entra_tentativo=SI; la confianza sobre la familia exacta de IA es media.</t>
+          <t>Caso clasificado en bloque '1-dudoso'. DUDA CENTRAL (¿IA real vs lógica de reglas?) RESUELTA hacia SI: la ficha técnica oficial de GEMA (Datys) lo describe como herramienta de análisis de grandes volúmenes de archivos con recuperación de información, clasificación por temáticas, OCR, agrupamiento de documentos similares y resumen automático extractivo -&gt; NLP/minería de texto/recuperación de información sobre el CONTENIDO, no mero conteo ni agrupación determinista trivial.</t>
         </is>
       </c>
     </row>
@@ -23355,7 +23355,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Limitación de acceso: WebFetch devolvió HTTP 403 en TODAS las URLs relevantes (Datys, Granma, Cubadebate, espirituano.gob.cu, OnCuba, Wikipedia, Resumen Latinoamericano) y el host de Datys no está en el allowlist para curl. El contenido y las citas se recuperaron vía WebSearch, que reprodujo el texto de forma consistente en varias fuentes oficiales y de prensa cubanas e independientes; no hubo verificación literal carácter a carácter sobre el HTML.</t>
+          <t>Persiste incertidumbre sobre la PROFUNDIDAD técnica del agrupamiento: las fuentes no confirman si usa ML/embeddings semánticos o similitud clásica de recuperación de información. En ambos escenarios se trata de procesamiento de texto sobre el contenido de los aportes, por lo que rol_IA=contenido y entra_tentativo=SI; la confianza sobre la familia exacta de IA es media.</t>
         </is>
       </c>
     </row>
@@ -23377,7 +23377,7 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Proceso de USO ÚNICO ya cerrado (febrero-abril 2022); no hay evidencia de actividad ni nuevas ediciones en 2026. estado_actividad='cerrado'. El Código entró en vigor en septiembre de 2022 tras referendo, pero el proceso participativo con IA finalizó en 2022.</t>
+          <t>Limitación de acceso: WebFetch devolvió HTTP 403 en TODAS las URLs relevantes (Datys, Granma, Cubadebate, espirituano.gob.cu, OnCuba, Wikipedia, Resumen Latinoamericano) y el host de Datys no está en el allowlist para curl. El contenido y las citas se recuperaron vía WebSearch, que reprodujo el texto de forma consistente en varias fuentes oficiales y de prensa cubanas e independientes; no hubo verificación literal carácter a carácter sobre el HTML.</t>
         </is>
       </c>
     </row>
@@ -23399,7 +23399,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>GEMA-CEN es la instancia de GEMA adaptada para el Consejo Electoral Nacional (CEN); el sufijo '-CEN' refiere al órgano, no a una variante técnica distinta documentada.</t>
+          <t>Proceso de USO ÚNICO ya cerrado (febrero-abril 2022); no hay evidencia de actividad ni nuevas ediciones en 2026. estado_actividad='cerrado'. El Código entró en vigor en septiembre de 2022 tras referendo, pero el proceso participativo con IA finalizó en 2022.</t>
         </is>
       </c>
     </row>
@@ -23421,7 +23421,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>tipo_proceso: se asignó 'Participación Digital' (se apoyó en plataformas/sistemas digitales y app de la UCI) y 'Referendos e Iniciativas Populares' (consulta popular legislativa vinculada a un referendo nacional). Etiquetado interpretativo; el núcleo es una consulta popular legislativa de iniciativa estatal.</t>
+          <t>GEMA-CEN es la instancia de GEMA adaptada para el Consejo Electoral Nacional (CEN); el sufijo '-CEN' refiere al órgano, no a una variante técnica distinta documentada.</t>
         </is>
       </c>
     </row>
@@ -23443,29 +23443,29 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Contexto político: diversas fuentes (elTOQUE, Voz y Voto, Washington Blade) cuestionan el carácter genuinamente participativo/garantista de la consulta ('debate guiado'). No afecta la elegibilidad técnica (sí hubo recogida de propuestas y uso de IA sobre su contenido), pero se registra como matiz de calidad democrática del proceso.</t>
+          <t>tipo_proceso: se asignó 'Participación Digital' (se apoyó en plataformas/sistemas digitales y app de la UCI) y 'Referendos e Iniciativas Populares' (consulta popular legislativa vinculada a un referendo nacional). Etiquetado interpretativo; el núcleo es una consulta popular legislativa de iniciativa estatal.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>TT-engagett-plataforma-go-vocal</t>
+          <t>CU-consulta-popular-codigo-de-las-familias</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>CU</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
+          <t>Consulta Popular Código de las Familias (GEMA-CEN / XISCOP)</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>[2a pasada DUDA-&gt;DUDA(lean NO)] Hallazgo NUEVO decisivo: la funcion de IA/NLP de Go Vocal (Sensemaking/AI Analysis) NO viene activa por defecto sino que DEPENDE DEL PLAN ('Access to this feature depends on your plan. Advanced Sensemaking with auto-insights is available in the Premium plan' - Go Vocal Support Base). Tras &gt;=14 busquedas/fetches dirigidos NO se halla NINGUNA evidencia de que la instancia de Trinidad (engage.gov.tt) active ni use ese analisis IA sobre el CONTENIDO de los aportes del NDTS: todo describe EngageTT como recolector (surveys/polls/Open Forum/ideas), uso de plataforma como formulario. Por eso usa_IA_en_proceso=no y rol_IA=no-usa. Se mantiene DUDA con LEAN NO por el unico cabo no verificable: la metodologia del PDF 'NDTS 2025 - Actionable Feedback &amp; Implementation Plan' (engage.gov.tt bloqueado a nivel de gateway del proxy, HTTP 403 policy denial), lo unico que podria voltear a SI. URL a revisar manualmente: https://engage.gov.tt/ideas/ndts-2025-actionable-feedback-implementation-plan</t>
+          <t>Contexto político: diversas fuentes (elTOQUE, Voz y Voto, Washington Blade) cuestionan el carácter genuinamente participativo/garantista de la consulta ('debate guiado'). No afecta la elegibilidad técnica (sí hubo recogida de propuestas y uso de IA sobre su contenido), pero se registra como matiz de calidad democrática del proceso.</t>
         </is>
       </c>
     </row>
@@ -23487,7 +23487,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>ELEGIBILIDAD (DUDA lean NO): proceso participativo genuino (consulta/planificacion nacional del NDTS 2024-2027, convocante gobierno nacional) sobre plataforma Go Vocal que TIENE IA/NLP de sensemaking pero solo en planes superiores (Premium), SIN evidencia de que la instancia TT active esa IA sobre el contenido de los aportes. Si se confirmara que NO se activa la IA -&gt; NO (no entra). Si el PDF de Actionable Feedback revelara analisis automatico del contenido por IA -&gt; SI.</t>
+          <t>[3a pasada amplia-&gt;DUDA(lean NO)] Busqueda AMPLIA (12+ busquedas/fetches EN/ES por canales diversos: documentacion Go Vocal/plan, proceso NDTS, MPAAI, Oxford Insights, prensa Caribe/LATAM) NO halla ninguna evidencia nueva de que engage.gov.tt (Trinidad) active/use IA/NLP (Sensemaking/AI Analysis) sobre el CONTENIDO de los aportes del NDTS. Al contrario, se refuerza el LEAN NO con 2 hallazgos NUEVOS: (1) Oxford Insights: 'The country's AI utilisation for citizens is concentrated in a robust Chatbot programme' (mas LLM de uso INTERNO) -&gt; la IA ciudadana de TT es el chatbot (AskNDTS/ANANSI), EXCLUIDO, no el analisis de aportes; (2) material MPAAI 2026 enmarca la IA en ANANSI (asistente de servicio publico) y encuestas de AI-readiness ('consolidated and reviewed'), sin mencion de Go Vocal Sensemaking ni de analisis IA de los aportes del NDTS. La IA de Go Vocal sigue confirmada como opcional/por plan ('Advanced Sensemaking with auto-insights is available in the Premium plan') y sin activacion confirmada en TT; no existe caso de cliente Go Vocal publicado para Trinidad (a diferencia de Cambridge/Viena). Persiste el UNICO cabo no verificable: metodologia del PDF 'NDTS 2025 - Actionable Feedback &amp; Implementation Plan' (engage.gov.tt = HTTP 403 policy denial en el gateway del proxy; ningun buscador expone el texto), lo unico que podria voltear a SI. Se mantiene DUDA(lean NO). URL a revisar manualmente: https://engage.gov.tt/ideas/ndts-2025-actionable-feedback-implementation-plan</t>
         </is>
       </c>
     </row>
@@ -23509,7 +23509,7 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>EXCLUSION explicita: AskNDTS es un chatbot/PWA de IA conversacional (FAQ sobre el NDTS), que segun el criterio (chatbot informativo/FAQ) NO cuenta como IA sobre el contenido de los aportes. Es la unica IA confirmada y desplegada en el ecosistema TT del NDTS.</t>
+          <t>[2a pasada DUDA-&gt;DUDA(lean NO)] Hallazgo NUEVO decisivo: la funcion de IA/NLP de Go Vocal (Sensemaking/AI Analysis) NO viene activa por defecto sino que DEPENDE DEL PLAN ('Access to this feature depends on your plan. Advanced Sensemaking with auto-insights is available in the Premium plan' - Go Vocal Support Base). Tras &gt;=14 busquedas/fetches dirigidos NO se halla NINGUNA evidencia de que la instancia de Trinidad (engage.gov.tt) active ni use ese analisis IA sobre el CONTENIDO de los aportes del NDTS: todo describe EngageTT como recolector (surveys/polls/Open Forum/ideas), uso de plataforma como formulario. Por eso usa_IA_en_proceso=no y rol_IA=no-usa. Se mantiene DUDA con LEAN NO por el unico cabo no verificable: la metodologia del PDF 'NDTS 2025 - Actionable Feedback &amp; Implementation Plan' (engage.gov.tt bloqueado a nivel de gateway del proxy, HTTP 403 policy denial), lo unico que podria voltear a SI. URL a revisar manualmente: https://engage.gov.tt/ideas/ndts-2025-actionable-feedback-implementation-plan</t>
         </is>
       </c>
     </row>
@@ -23531,7 +23531,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMACION TECNICA: engage.gov.tt corre sobre Go Vocal (antes CitizenLab), confirmado por la ruta interna 'projects/e-democracy-govocal-internal' indexada por buscadores.</t>
+          <t>ELEGIBILIDAD (DUDA lean NO): proceso participativo genuino (consulta/planificacion nacional del NDTS 2024-2027, convocante gobierno nacional) sobre plataforma Go Vocal que TIENE IA/NLP de sensemaking pero solo en planes superiores (Premium), SIN evidencia de que la instancia TT active esa IA sobre el contenido de los aportes. Si se confirmara que NO se activa la IA -&gt; NO (no entra). Si el PDF de Actionable Feedback revelara analisis automatico del contenido por IA -&gt; SI.</t>
         </is>
       </c>
     </row>
@@ -23553,7 +23553,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>FUENTES: engage.gov.tt, govocal.com y support.govocal.com devuelven HTTP 403 a WebFetch; ademas el proxy registra 'connect_rejected / gateway answered 403 to CONNECT (policy denial or upstream failure)' para host engage.gov.tt:443 (bloqueo a nivel de gateway), y el intento de descarga por curl tambien fue rechazado en el CONNECT (403). mdt.gov.tt da ENOTFOUND (DNS) -dominio del ministerio previo absorbido tras la fusion en MPAAI en may-2025-. Todo el contenido y las citas se recuperaron de forma convergente via WebSearch (&gt;=14 consultas/fetches en total). Confianza MEDIA: la decision lean NO se apoya en (a) que la IA de Go Vocal es opcional/por plan y (b) ausencia total de evidencia de activacion en TT; el unico residuo de duda es el PDF no recuperable.</t>
+          <t>EXCLUSION explicita: AskNDTS es un chatbot/PWA de IA conversacional (FAQ sobre el NDTS), que segun el criterio (chatbot informativo/FAQ) NO cuenta como IA sobre el contenido de los aportes. Es la unica IA confirmada y desplegada en el ecosistema TT del NDTS.</t>
         </is>
       </c>
     </row>
@@ -23575,7 +23575,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>DESARROLLADOR: Go Vocal (antes CitizenLab) es una empresa fundada en 2015 con sede en Belgica (Privado, origen Internacional). Convocante/operador del proceso = gobierno nacional de Trinidad y Tobago (Ministry of Digital Transformation / MPAAI), con colaboracion del BID/IDB.</t>
+          <t>CONFIRMACION TECNICA: engage.gov.tt corre sobre Go Vocal (antes CitizenLab), confirmado por la ruta interna 'projects/e-democracy-govocal-internal' indexada por buscadores.</t>
         </is>
       </c>
     </row>
@@ -23597,51 +23597,51 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>CONTEXTO INSTITUCIONAL: el 23-may-2025 el Ministry of Public Administration y el Ministry of Digital Transformation se fusionaron en el Ministry of Public Administration and Artificial Intelligence (MPAAI); engage.gov.tt ahora figura bajo MPAAI.</t>
+          <t>FUENTES: engage.gov.tt, govocal.com y support.govocal.com devuelven HTTP 403 a WebFetch; ademas el proxy registra 'connect_rejected / gateway answered 403 to CONNECT (policy denial or upstream failure)' para host engage.gov.tt:443 (bloqueo a nivel de gateway), y el intento de descarga por curl tambien fue rechazado en el CONNECT (403). mdt.gov.tt da ENOTFOUND (DNS) -dominio del ministerio previo absorbido tras la fusion en MPAAI en may-2025-. Todo el contenido y las citas se recuperaron de forma convergente via WebSearch (&gt;=14 consultas/fetches en total). Confianza MEDIA: la decision lean NO se apoya en (a) que la IA de Go Vocal es opcional/por plan y (b) ausencia total de evidencia de activacion en TT; el unico residuo de duda es el PDF no recuperable.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>VE-plan-de-la-patria-7-transformaciones-ia</t>
+          <t>TT-engagett-plataforma-go-vocal</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>VE</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Plan de la Patria 7 Transformaciones (7T) - IA y Big Data en la sistematización de propuestas de la Consulta Popular</t>
+          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>[2ª pasada DUDA→NO] Sin corroboración técnica independiente. Tras 6-10 búsquedas/fetches dirigidos (ES/EN; proveedor, académico, documento técnico, MINCYT/MPPP) NO se halló ninguna fuente independiente que confirme IA/NLP/ML procesando el CONTENIDO de las propuestas. La 2ª pasada además RECUPERÓ la metodología oficial de sistematización HUMANA (sistema web hagamospatria.org.ve, transcriptores, revisión 'una por una' por el equipo con herramientas informáticas de clasificación en 4 categorías, relator que valida con participantes, 3 niveles de agregación, SIG), que es la función verificable. La afirmación estatal 'IA+Big Data procesaron 500.000+ propuestas para generar los algoritmos' sigue siendo retórica política sin modelo/proveedor/técnica y contradice la cifra robusta de 34.491. Veredicto binario: NO. Confianza BAJA. Dato verificable conservado: 34.491 propuestas sistematizadas por relatores humanos + herramientas de clasificación + SIG. URL de prensa estatal en gaps para revisión manual.</t>
+          <t>DESARROLLADOR: Go Vocal (antes CitizenLab) es una empresa fundada en 2015 con sede en Belgica (Privado, origen Internacional). Convocante/operador del proceso = gobierno nacional de Trinidad y Tobago (Ministry of Digital Transformation / MPAAI), con colaboracion del BID/IDB.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>VE-plan-de-la-patria-7-transformaciones-ia</t>
+          <t>TT-engagett-plataforma-go-vocal</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>VE</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Plan de la Patria 7 Transformaciones (7T) - IA y Big Data en la sistematización de propuestas de la Consulta Popular</t>
+          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_PRENSA_ESTATAL: la afirmación central (IA+Big Data procesaron 500.000+ propuestas) proviene de medios del Estado (Correo del Orinoco, MINCYT, Cendit, FEVP, MPPRE, todos .gob.ve) y mirrors oficialistas. Es AFIRMACIÓN POLÍTICA, no evidencia técnica. No se halló corroboración independiente (proveedor, paper, académico). Tratar con escepticismo alto.</t>
+          <t>CONTEXTO INSTITUCIONAL: el 23-may-2025 el Ministry of Public Administration y el Ministry of Digital Transformation se fusionaron en el Ministry of Public Administration and Artificial Intelligence (MPAAI); engage.gov.tt ahora figura bajo MPAAI.</t>
         </is>
       </c>
     </row>
@@ -23663,7 +23663,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_CONTRADICCION_CIFRAS: la cifra estatal de IA ('más de 500.000 propuestas') contradice la cifra metodológica oficial verificable de 34.491 propuestas (con 33.780 relatores y 3,4 M de participantes). Esta discrepancia de un orden de magnitud refuerza que '500.000' es retórica y que el dato robusto es 34.491.</t>
+          <t>[2ª pasada DUDA→NO] Sin corroboración técnica independiente. Tras 6-10 búsquedas/fetches dirigidos (ES/EN; proveedor, académico, documento técnico, MINCYT/MPPP) NO se halló ninguna fuente independiente que confirme IA/NLP/ML procesando el CONTENIDO de las propuestas. La 2ª pasada además RECUPERÓ la metodología oficial de sistematización HUMANA (sistema web hagamospatria.org.ve, transcriptores, revisión 'una por una' por el equipo con herramientas informáticas de clasificación en 4 categorías, relator que valida con participantes, 3 niveles de agregación, SIG), que es la función verificable. La afirmación estatal 'IA+Big Data procesaron 500.000+ propuestas para generar los algoritmos' sigue siendo retórica política sin modelo/proveedor/técnica y contradice la cifra robusta de 34.491. Veredicto binario: NO. Confianza BAJA. Dato verificable conservado: 34.491 propuestas sistematizadas por relatores humanos + herramientas de clasificación + SIG. URL de prensa estatal en gaps para revisión manual.</t>
         </is>
       </c>
     </row>
@@ -23685,7 +23685,7 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_EJE_VS_HERRAMIENTA: 'incluir la IA en el Plan de las 7T' = IA como EJE TEMÁTICO/PRIORIDAD del plan de gobierno (de ahí el Plan Nacional de IA, Ley de IA y Código de Ética feb-2026), NO una herramienta que procesa los aportes de la consulta. La coletilla estatal 'para generar los algoritmos' confirma que la IA es el PRODUCTO/objetivo de esa agenda, no una herramienta aplicada a los aportes. Por la regla del índice, eje temático ≠ elegibilidad. Base de la calificación NO.</t>
+          <t>ALERTA_PRENSA_ESTATAL: la afirmación central (IA+Big Data procesaron 500.000+ propuestas) proviene de medios del Estado (Correo del Orinoco, MINCYT, Cendit, FEVP, MPPRE, todos .gob.ve) y mirrors oficialistas. Es AFIRMACIÓN POLÍTICA, no evidencia técnica. No se halló corroboración independiente (proveedor, paper, académico). Tratar con escepticismo alto.</t>
         </is>
       </c>
     </row>
@@ -23707,7 +23707,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_PROCESAMIENTO_HUMANO+SIG: la evidencia técnica verificable (metodología oficial del Plan 7T) indica que las 34.491 propuestas fueron cargadas/transcritas/sistematizadas por 33.780 RELATORES HUMANOS en el sistema web hagamospatria.org.ve, revisadas 'una por una' y clasificadas en cuatro categorías con apoyo de herramientas informáticas, validadas con los participantes, agregadas en tres niveles, con georreferenciación vía SIG y QR del Carnet de la Patria. Esto es procesamiento humano + clasificación informática + sistema de información geográfica, NO IA de análisis de contenido.</t>
+          <t>ALERTA_CONTRADICCION_CIFRAS: la cifra estatal de IA ('más de 500.000 propuestas') contradice la cifra metodológica oficial verificable de 34.491 propuestas (con 33.780 relatores y 3,4 M de participantes). Esta discrepancia de un orden de magnitud refuerza que '500.000' es retórica y que el dato robusto es 34.491.</t>
         </is>
       </c>
     </row>
@@ -23729,7 +23729,7 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_FUENTES_403: todas las URLs .gob.ve (correodelorinoco, mincyt, cendit, fevp, mppre, mppp, noticias.patria), es.wikipedia y la copia archive.org del PDF del Plan 7T devolvieron HTTP 403 a WebFetch (en http y https; el proxy de egreso confirma 403 de política). Las citas se recuperaron vía snippets de WebSearch que indexan esas mismas URLs. Conviene verificación manual directa.</t>
+          <t>ALERTA_EJE_VS_HERRAMIENTA: 'incluir la IA en el Plan de las 7T' = IA como EJE TEMÁTICO/PRIORIDAD del plan de gobierno (de ahí el Plan Nacional de IA, Ley de IA y Código de Ética feb-2026), NO una herramienta que procesa los aportes de la consulta. La coletilla estatal 'para generar los algoritmos' confirma que la IA es el PRODUCTO/objetivo de esa agenda, no una herramienta aplicada a los aportes. Por la regla del índice, eje temático ≠ elegibilidad. Base de la calificación NO.</t>
         </is>
       </c>
     </row>
@@ -23751,7 +23751,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_CONFIANZA_BAJA: confianza=BAJA por basarse en una sola narrativa estatal repetida en varios portales oficialistas (no fuentes independientes), sin corroboración técnica y con contradicción de cifras. El veredicto NO se apoya en AUSENCIA de evidencia de IA + PRESENCIA de evidencia de procesamiento humano; no elevar la confianza sin un documento metodológico/técnico del MPPP o del MINCYT que aún no existe.</t>
+          <t>ALERTA_PROCESAMIENTO_HUMANO+SIG: la evidencia técnica verificable (metodología oficial del Plan 7T) indica que las 34.491 propuestas fueron cargadas/transcritas/sistematizadas por 33.780 RELATORES HUMANOS en el sistema web hagamospatria.org.ve, revisadas 'una por una' y clasificadas en cuatro categorías con apoyo de herramientas informáticas, validadas con los participantes, agregadas en tres niveles, con georreferenciación vía SIG y QR del Carnet de la Patria. Esto es procesamiento humano + clasificación informática + sistema de información geográfica, NO IA de análisis de contenido.</t>
         </is>
       </c>
     </row>
@@ -23773,51 +23773,51 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>ALERTA_VERIFICACION_MANUAL: verificación manual residual recomendada con (1) MPPP — documento metodológico del Plan 7T (confirma sistematización humana); (2) MINCYT — si el Plan Nacional de IA llegara a documentar algún componente real aplicado a los aportes de la consulta; (3) PDF del Plan de la Patria 7T para lectura verbatim. URLs en gaps. A la fecha (jun-2026) no hay tal documento técnico.</t>
+          <t>ALERTA_FUENTES_403: todas las URLs .gob.ve (correodelorinoco, mincyt, cendit, fevp, mppre, mppp, noticias.patria), es.wikipedia y la copia archive.org del PDF del Plan 7T devolvieron HTTP 403 a WebFetch (en http y https; el proxy de egreso confirma 403 de política). Las citas se recuperaron vía snippets de WebSearch que indexan esas mismas URLs. Conviene verificación manual directa.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>CL-EXC-ucampus</t>
+          <t>VE-plan-de-la-patria-7-transformaciones-ia</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>VE</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Plataforma UCampus - participación 2023 (proceso constitucional)</t>
+          <t>Plan de la Patria 7 Transformaciones (7T) - IA y Big Data en la sistematización de propuestas de la Consulta Popular</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>DECISIÓN: MANTENER EXCLUIDO (entra=NO). No se confirma IA sobre el CONTENIDO de los aportes ciudadanos en la plataforma UCampus 2023. UCampus operó como gestor tecnológico (recepción de Audiencias Públicas e Iniciativas Populares de Norma: solicitar audiencia, revisar artículos, proponer enmiendas, recolectar 10.000 firmas con ClaveÚnica). La sistematización analítica fue CUALITATIVA, encabezada por académicos de derecho constitucional y ciencias sociales.</t>
+          <t>ALERTA_CONFIANZA_BAJA: confianza=BAJA por basarse en una sola narrativa estatal repetida en varios portales oficialistas (no fuentes independientes), sin corroboración técnica y con contradicción de cifras. El veredicto NO se apoya en AUSENCIA de evidencia de IA + PRESENCIA de evidencia de procesamiento humano; no elevar la confianza sin un documento metodológico/técnico del MPPP o del MINCYT que aún no existe.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>CL-EXC-ucampus</t>
+          <t>VE-plan-de-la-patria-7-transformaciones-ia</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>VE</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Plataforma UCampus - participación 2023 (proceso constitucional)</t>
+          <t>Plan de la Patria 7 Transformaciones (7T) - IA y Big Data en la sistematización de propuestas de la Consulta Popular</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>RIESGO DE FALSO POSITIVO EVITADO: durante el proceso constitucional 2023 sí circularon herramientas de IA (Constitucion.AI de kemeny.studio, Discolab/UDD, ChatBot Constitucional U.Central), pero TODAS operaron sobre el TEXTO DE LA PROPUESTA constitucional para facilitar su comprensión a la ciudadanía -no sobre los aportes ciudadanos- y son iniciativas INDEPENDIENTES sin vínculo oficial con UCampus ni con la Secretaría de Participación. No deben confundirse con el caso UCampus.</t>
+          <t>ALERTA_VERIFICACION_MANUAL: verificación manual residual recomendada con (1) MPPP — documento metodológico del Plan 7T (confirma sistematización humana); (2) MINCYT — si el Plan Nacional de IA llegara a documentar algún componente real aplicado a los aportes de la consulta; (3) PDF del Plan de la Patria 7T para lectura verbatim. URLs en gaps. A la fecha (jun-2026) no hay tal documento técnico.</t>
         </is>
       </c>
     </row>
@@ -23839,7 +23839,7 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>CONTRASTE CON CABILDOS 2016: el motivo de revisión era confirmar si, como en los cabildos del proceso constituyente 2016 (donde hubo análisis NLP de aportes), UCampus 2023 aplicó NLP a los aportes. La evidencia encontrada NO lo confirma; el proceso 2023 sistematizó cualitativamente. Si el informe oficial (PDF, hoy 403) revelara procesamiento automático/NLP de los aportes, el caso pasaría a DUDA y podría reingresar.</t>
+          <t>DECISIÓN: MANTENER EXCLUIDO (entra=NO). No se confirma IA sobre el CONTENIDO de los aportes ciudadanos en la plataforma UCampus 2023. UCampus operó como gestor tecnológico (recepción de Audiencias Públicas e Iniciativas Populares de Norma: solicitar audiencia, revisar artículos, proponer enmiendas, recolectar 10.000 firmas con ClaveÚnica). La sistematización analítica fue CUALITATIVA, encabezada por académicos de derecho constitucional y ciencias sociales.</t>
         </is>
       </c>
     </row>
@@ -23861,7 +23861,7 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>FUENTES 403: las URLs institucionales clave (uchile.cl, ingenieria.uchile.cl, varias de ucampus.cl, procesoconstitucional.cl, secretariadeparticipacion.cl y el PDF del informe) devolvieron HTTP 403 tanto a WebFetch como a curl a través del proxy del entorno. El contenido y las citas verbatim se recuperaron de manera consistente vía WebSearch sobre esas mismas URLs. Confianza MEDIA: la ausencia de IA sobre el contenido es coherente en todas las fuentes accesibles, pero el informe oficial completo no pudo leerse directamente y queda en gaps para verificación manual.</t>
+          <t>RIESGO DE FALSO POSITIVO EVITADO: durante el proceso constitucional 2023 sí circularon herramientas de IA (Constitucion.AI de kemeny.studio, Discolab/UDD, ChatBot Constitucional U.Central), pero TODAS operaron sobre el TEXTO DE LA PROPUESTA constitucional para facilitar su comprensión a la ciudadanía -no sobre los aportes ciudadanos- y son iniciativas INDEPENDIENTES sin vínculo oficial con UCampus ni con la Secretaría de Participación. No deben confundirse con el caso UCampus.</t>
         </is>
       </c>
     </row>
@@ -23883,7 +23883,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>tipo_proceso: se clasifica como 'Participación Digital' + 'Referendos e Iniciativas Populares' porque los dos mecanismos operados por UCampus fueron Audiencias Públicas e Iniciativa Popular de Norma (mecanismo de iniciativa popular con umbral de 10.000 firmas).</t>
+          <t>CONTRASTE CON CABILDOS 2016: el motivo de revisión era confirmar si, como en los cabildos del proceso constituyente 2016 (donde hubo análisis NLP de aportes), UCampus 2023 aplicó NLP a los aportes. La evidencia encontrada NO lo confirma; el proceso 2023 sistematizó cualitativamente. Si el informe oficial (PDF, hoy 403) revelara procesamiento automático/NLP de los aportes, el caso pasaría a DUDA y podría reingresar.</t>
         </is>
       </c>
     </row>
@@ -23905,51 +23905,51 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>nivel_consolidacion=2 (puntual): única edición del proceso constitucional 2023; UCampus participó en ese proceso específico, sin ediciones recurrentes de esta plataforma de participación constitucional.</t>
+          <t>FUENTES 403: las URLs institucionales clave (uchile.cl, ingenieria.uchile.cl, varias de ucampus.cl, procesoconstitucional.cl, secretariadeparticipacion.cl y el PDF del informe) devolvieron HTTP 403 tanto a WebFetch como a curl a través del proxy del entorno. El contenido y las citas verbatim se recuperaron de manera consistente vía WebSearch sobre esas mismas URLs. Confianza MEDIA: la ausencia de IA sobre el contenido es coherente en todas las fuentes accesibles, pero el informe oficial completo no pudo leerse directamente y queda en gaps para verificación manual.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>CO-EXC-asamblea-itinerante</t>
+          <t>CL-EXC-ucampus</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Asamblea Ciudadana Itinerante del Concejo de Bogotá</t>
+          <t>Plataforma UCampus - participación 2023 (proceso constitucional)</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Posible confusion entre dos procesos distintos: (1) 'Asamblea Ciudadana Itinerante del Concejo de Bogota' (Concejo via DemoLab, 2020/2021/2023) y (2) 'Asambleas Deliberativas #SumemosVoces' (Alcaldia/Secretaria Distrital de Planeacion, 2024-2027). No deben fusionarse.</t>
+          <t>tipo_proceso: se clasifica como 'Participación Digital' + 'Referendos e Iniciativas Populares' porque los dos mecanismos operados por UCampus fueron Audiencias Públicas e Iniciativa Popular de Norma (mecanismo de iniciativa popular con umbral de 10.000 firmas).</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>CO-EXC-asamblea-itinerante</t>
+          <t>CL-EXC-ucampus</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Asamblea Ciudadana Itinerante del Concejo de Bogotá</t>
+          <t>Plataforma UCampus - participación 2023 (proceso constitucional)</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>La relacion entre el caso y la IA es solo tematica (ambos tocan el POT). El estudio 'Factibilidad de IA... caso del POT' es investigacion academica de aceptacion de una herramienta PROPUESTA, no un sistema de IA operando dentro de la Asamblea.</t>
+          <t>nivel_consolidacion=2 (puntual): única edición del proceso constitucional 2023; UCampus participó en ese proceso específico, sin ediciones recurrentes de esta plataforma de participación constitucional.</t>
         </is>
       </c>
     </row>
@@ -23971,14 +23971,14 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Todas las fuentes primarias devolvieron 403 a WebFetch; la verificacion se apoyo en snippets de WebSearch. Confianza limitada a MEDIA por ausencia de verbatim directo del HTML fuente.</t>
+          <t>Posible confusion entre dos procesos distintos: (1) 'Asamblea Ciudadana Itinerante del Concejo de Bogota' (Concejo via DemoLab, 2020/2021/2023) y (2) 'Asambleas Deliberativas #SumemosVoces' (Alcaldia/Secretaria Distrital de Planeacion, 2024-2027). No deben fusionarse.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>CO-EXC-procuraduria</t>
+          <t>CO-EXC-asamblea-itinerante</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -23988,19 +23988,19 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Mini-Public del diálogo social de la Procuraduría</t>
+          <t>Asamblea Ciudadana Itinerante del Concejo de Bogotá</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>DECISIÓN: se MANTIENE EXCLUIDO (entra=NO), confirmando la exclusión 2025. El proceso es ELEGIBLE por su naturaleza (mini-público / diálogo social convocado por la Procuraduría y facilitado por ideemos), pero NO hay evidencia de IA sobre el CONTENIDO de los aportes ciudadanos, que es el requisito de reingreso. No es DUDA: es ausencia de evidencia, no indicio no concluyente.</t>
+          <t>La relacion entre el caso y la IA es solo tematica (ambos tocan el POT). El estudio 'Factibilidad de IA... caso del POT' es investigacion academica de aceptacion de una herramienta PROPUESTA, no un sistema de IA operando dentro de la Asamblea.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>CO-EXC-procuraduria</t>
+          <t>CO-EXC-asamblea-itinerante</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -24010,12 +24010,12 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Mini-Public del diálogo social de la Procuraduría</t>
+          <t>Asamblea Ciudadana Itinerante del Concejo de Bogotá</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>ACCESO A FUENTES: la URL original del caso (ideemos.org/mini-public-del-dialogo-social-de-la-procuraduria/) y todo ideemos.org devuelven HTTP 403 a WebFetch; el micrositio escuelasdialogopgn.com falla por DNS (ENOTFOUND) vía proxy; web.archive.org está bloqueado para esta herramienta. Toda la información se reconstruyó a partir de snippets de WebSearch, no de transcripción directa de las páginas renderizadas; por ello confianza MEDIA. Las citas verbatim provienen de los extractos devueltos por WebSearch sobre esas mismas URLs.</t>
+          <t>Todas las fuentes primarias devolvieron 403 a WebFetch; la verificacion se apoyo en snippets de WebSearch. Confianza limitada a MEDIA por ausencia de verbatim directo del HTML fuente.</t>
         </is>
       </c>
     </row>
@@ -24037,7 +24037,7 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>IA DE LA PROCURADURÍA ES AJENA AL PROCESO: las menciones reales de IA en la Procuraduría se refieren a (a) herramienta de consulta con IA para la Guía Disciplinaria (asuntos disciplinarios, nov-2025) y (b) preparación frente a redes, algoritmos e IA / desinformación para proteger la democracia (foro Semana). Ninguna procesa los aportes del mini-público / diálogo social. No deben confundirse con IA sobre el contenido de las contribuciones ciudadanas.</t>
+          <t>DECISIÓN: se MANTIENE EXCLUIDO (entra=NO), confirmando la exclusión 2025. El proceso es ELEGIBLE por su naturaleza (mini-público / diálogo social convocado por la Procuraduría y facilitado por ideemos), pero NO hay evidencia de IA sobre el CONTENIDO de los aportes ciudadanos, que es el requisito de reingreso. No es DUDA: es ausencia de evidencia, no indicio no concluyente.</t>
         </is>
       </c>
     </row>
@@ -24059,7 +24059,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>tipo_convocante: la Procuraduría General de la Nación se clasifica como 'otra institución pública' (órgano de control autónomo, no es gobierno nacional del ejecutivo ni gobierno local). Facilitador ideemos = sociedad civil (laboratorio de innovación democrática, SAS, Bogotá). tipo_organizacion=Público (proceso convocado por institución pública).</t>
+          <t>ACCESO A FUENTES: la URL original del caso (ideemos.org/mini-public-del-dialogo-social-de-la-procuraduria/) y todo ideemos.org devuelven HTTP 403 a WebFetch; el micrositio escuelasdialogopgn.com falla por DNS (ENOTFOUND) vía proxy; web.archive.org está bloqueado para esta herramienta. Toda la información se reconstruyó a partir de snippets de WebSearch, no de transcripción directa de las páginas renderizadas; por ello confianza MEDIA. Las citas verbatim provienen de los extractos devueltos por WebSearch sobre esas mismas URLs.</t>
         </is>
       </c>
     </row>
@@ -24081,14 +24081,14 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>RECOMENDACIÓN: si en una revisión posterior se logra acceso directo (o copia archivada) a la página de ideemos del caso y/o a informes metodológicos de las Escuelas de Diálogo PGN, verificar específicamente si la relatoría o sistematización de los aportes usa NLP/LLM. Hasta entonces, mantener excluido.</t>
+          <t>IA DE LA PROCURADURÍA ES AJENA AL PROCESO: las menciones reales de IA en la Procuraduría se refieren a (a) herramienta de consulta con IA para la Guía Disciplinaria (asuntos disciplinarios, nov-2025) y (b) preparación frente a redes, algoritmos e IA / desinformación para proteger la democracia (foro Semana). Ninguna procesa los aportes del mini-público / diálogo social. No deben confundirse con IA sobre el contenido de las contribuciones ciudadanas.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>CO-EXC-paqueveas</t>
+          <t>CO-EXC-procuraduria</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -24098,19 +24098,19 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Pa' que veás (Cali)</t>
+          <t>Mini-Public del diálogo social de la Procuraduría</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Analogia con dIAra NO se sostiene: dIAra aplica IA al contenido de quejas ciudadanas; 'Pa' que veas' es un monitor de inversion publica (MapaInversiones del BID) que visualiza gasto/contratos, sin IA sobre aportes ciudadanos.</t>
+          <t>tipo_convocante: la Procuraduría General de la Nación se clasifica como 'otra institución pública' (órgano de control autónomo, no es gobierno nacional del ejecutivo ni gobierno local). Facilitador ideemos = sociedad civil (laboratorio de innovación democrática, SAS, Bogotá). tipo_organizacion=Público (proceso convocado por institución pública).</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>CO-EXC-paqueveas</t>
+          <t>CO-EXC-procuraduria</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -24120,12 +24120,12 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Pa' que veás (Cali)</t>
+          <t>Mini-Public del diálogo social de la Procuraduría</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Posible confusion por co-mencion: el boletin 'Cali, lider en IA' lista 'Pa' que veas' junto a chatbots y analisis predictivo, pero el monitor solo se encuadra en 'gestion eficiente de datos / seguimiento a la inversion publica'. Los usos de IA (chatbots de consulta, prediccion de deslizamientos/dengue/seguridad) son iniciativas SEPARADAS del ecosistema smart-city de Cali.</t>
+          <t>RECOMENDACIÓN: si en una revisión posterior se logra acceso directo (o copia archivada) a la página de ideemos del caso y/o a informes metodológicos de las Escuelas de Diálogo PGN, verificar específicamente si la relatoría o sistematización de los aportes usa NLP/LLM. Hasta entonces, mantener excluido.</t>
         </is>
       </c>
     </row>
@@ -24147,7 +24147,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Funcionalidades de reportes ciudadanos / alertas de irregularidades / fotografias estan anunciadas como evolucion FUTURA, no como capacidad actual; no procesadas por IA hasta donde documentan las fuentes.</t>
+          <t>Analogia con dIAra NO se sostiene: dIAra aplica IA al contenido de quejas ciudadanas; 'Pa' que veas' es un monitor de inversion publica (MapaInversiones del BID) que visualiza gasto/contratos, sin IA sobre aportes ciudadanos.</t>
         </is>
       </c>
     </row>
@@ -24169,14 +24169,14 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Todas las fuentes primarias devolvieron 403 a WebFetch; la verificacion se apoyo en snippets de WebSearch. Pese a ello, la convergencia de &gt;=2 fuentes independientes (BID + Alcaldia + prensa) sobre la naturaleza de dashboard sostiene confianza ALTA para la decision de exclusion.</t>
+          <t>Posible confusion por co-mencion: el boletin 'Cali, lider en IA' lista 'Pa' que veas' junto a chatbots y analisis predictivo, pero el monitor solo se encuadra en 'gestion eficiente de datos / seguimiento a la inversion publica'. Los usos de IA (chatbots de consulta, prediccion de deslizamientos/dengue/seguridad) son iniciativas SEPARADAS del ecosistema smart-city de Cali.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>CO-EXC-ilabs</t>
+          <t>CO-EXC-paqueveas</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -24186,19 +24186,19 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>iLabs - Laboratorios de Inteligencia Colectiva (Ideemos)</t>
+          <t>Pa' que veás (Cali)</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>ELEGIBILIDAD (motivo de exclusión 2025 confirmado): la única mención de IA/ML está en un listado de técnicas para COMPRENDER el problema (diagnóstico), separada de las técnicas de deliberación (mini-públicos). No hay evidencia de IA sobre el CONTENIDO de los aportes ciudadanos. Por la regla de reingreso =&gt; entra_tentativo=NO. No se eleva a DUDA por ser mención genérica de etapa de diagnóstico sin indicio concreto de procesamiento de contenido deliberativo.</t>
+          <t>Funcionalidades de reportes ciudadanos / alertas de irregularidades / fotografias estan anunciadas como evolucion FUTURA, no como capacidad actual; no procesadas por IA hasta donde documentan las fuentes.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>CO-EXC-ilabs</t>
+          <t>CO-EXC-paqueveas</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -24208,12 +24208,12 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>iLabs - Laboratorios de Inteligencia Colectiva (Ideemos)</t>
+          <t>Pa' que veás (Cali)</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>FUENTES: todas las URLs de ideemos.org y participedia.net devuelven HTTP 403 a WebFetch; el contenido y las citas se recuperaron de forma convergente mediante WebSearch (6 consultas en ES/EN sobre las mismas URLs). Las citas verbatim son reconstrucciones del texto devuelto por los snippets de WebSearch, no transcripción directa de la página renderizada; por ello confianza MEDIA (no ALTA pese a múltiples consultas convergentes sobre la fuente primaria).</t>
+          <t>Todas las fuentes primarias devolvieron 403 a WebFetch; la verificacion se apoyo en snippets de WebSearch. Pese a ello, la convergencia de &gt;=2 fuentes independientes (BID + Alcaldia + prensa) sobre la naturaleza de dashboard sostiene confianza ALTA para la decision de exclusion.</t>
         </is>
       </c>
     </row>
@@ -24235,7 +24235,7 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>ALCANCE: la 'IA' de iLabs es metodología de diagnóstico/inteligencia colectiva, no procesamiento automatizado de los aportes deliberativos. Si en una edición concreta apareciera evidencia de NLP/ML sobre las transcripciones de los mini-públicos, el caso debería reevaluarse a DUDA o SI.</t>
+          <t>ELEGIBILIDAD (motivo de exclusión 2025 confirmado): la única mención de IA/ML está en un listado de técnicas para COMPRENDER el problema (diagnóstico), separada de las técnicas de deliberación (mini-públicos). No hay evidencia de IA sobre el CONTENIDO de los aportes ciudadanos. Por la regla de reingreso =&gt; entra_tentativo=NO. No se eleva a DUDA por ser mención genérica de etapa de diagnóstico sin indicio concreto de procesamiento de contenido deliberativo.</t>
         </is>
       </c>
     </row>
@@ -24257,7 +24257,7 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>DESARROLLADOR/CONVOCANTE: Ideemos es una S.A.S. colombiana de innovación democrática que actúa como sociedad civil/consultoría; no es un proveedor de IA con producto nombrado. tipo_desarrollador_IA se marca 'Sociedad Civil' por defecto (la IA no es un sistema propio identificado). origen_desarrollador 'Nacional' (Colombia).</t>
+          <t>FUENTES: todas las URLs de ideemos.org y participedia.net devuelven HTTP 403 a WebFetch; el contenido y las citas se recuperaron de forma convergente mediante WebSearch (6 consultas en ES/EN sobre las mismas URLs). Las citas verbatim son reconstrucciones del texto devuelto por los snippets de WebSearch, no transcripción directa de la página renderizada; por ello confianza MEDIA (no ALTA pese a múltiples consultas convergentes sobre la fuente primaria).</t>
         </is>
       </c>
     </row>
@@ -24279,68 +24279,68 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>etapas_uso_IA se marca ['Planificación','Análisis'] referido al uso declarado de IA en la fase de COMPRENSIÓN/diagnóstico del problema (no en el análisis de los aportes), para reflejar dónde Ideemos ubica la IA; esto NO implica que califique para reingreso.</t>
+          <t>ALCANCE: la 'IA' de iLabs es metodología de diagnóstico/inteligencia colectiva, no procesamiento automatizado de los aportes deliberativos. Si en una edición concreta apareciera evidencia de NLP/ML sobre las transcripciones de los mini-públicos, el caso debería reevaluarse a DUDA o SI.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>BO-bolivia-conversa</t>
+          <t>CO-EXC-ilabs</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Bolivia Conversa</t>
+          <t>iLabs - Laboratorios de Inteligencia Colectiva (Ideemos)</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>DESARROLLADOR/CONVOCANTE: Ideemos es una S.A.S. colombiana de innovación democrática que actúa como sociedad civil/consultoría; no es un proveedor de IA con producto nombrado. tipo_desarrollador_IA se marca 'Sociedad Civil' por defecto (la IA no es un sistema propio identificado). origen_desarrollador 'Nacional' (Colombia).</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>BO-bolivia-conversa</t>
+          <t>CO-EXC-ilabs</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>BO</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Bolivia Conversa</t>
+          <t>iLabs - Laboratorios de Inteligencia Colectiva (Ideemos)</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>etapas_uso_IA se marca ['Planificación','Análisis'] referido al uso declarado de IA en la fase de COMPRENSIÓN/diagnóstico del problema (no en el análisis de los aportes), para reflejar dónde Ideemos ubica la IA; esto NO implica que califique para reingreso.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>BR-colab</t>
+          <t>BO-bolivia-conversa</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>BO</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Colab</t>
+          <t>Bolivia Conversa</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
@@ -24352,22 +24352,22 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>BR-colab</t>
+          <t>BO-bolivia-conversa</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>BO</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>Colab</t>
+          <t>Bolivia Conversa</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Plataforma desde 2013; posible nivel 3 con evidencia de recurrencia</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -24389,14 +24389,14 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>BR-participact-brasil</t>
+          <t>BR-colab</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -24406,19 +24406,19 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>ParticipACT Brasil</t>
+          <t>Colab</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>recodificación 2026: Plataforma desde 2013; posible nivel 3 con evidencia de recurrencia</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>BR-participact-brasil</t>
+          <t>BR-colab</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -24428,12 +24428,12 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>ParticipACT Brasil</t>
+          <t>Colab</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Convocante ambiguo: universidad vs sociedad civil</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -24455,14 +24455,14 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>BR-plan-plurianual-de-la-ciudad-de-natal</t>
+          <t>BR-participact-brasil</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -24472,19 +24472,19 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>Plan Plurianual de la ciudad de Natal</t>
+          <t>ParticipACT Brasil</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
+          <t>recodificación 2026: Convocante ambiguo: universidad vs sociedad civil</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>BR-plan-plurianual-de-la-ciudad-de-natal</t>
+          <t>BR-participact-brasil</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -24494,7 +24494,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>Plan Plurianual de la ciudad de Natal</t>
+          <t>ParticipACT Brasil</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -24506,7 +24506,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>BR-portal-e-cidadania-marcado-automatico-de</t>
+          <t>BR-plan-plurianual-de-la-ciudad-de-natal</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -24516,7 +24516,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>Portal e-Cidadania: Marcado automático de respuestas ciudadanas en videos de audiencias públicas</t>
+          <t>Plan Plurianual de la ciudad de Natal</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -24528,7 +24528,7 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>BR-portal-e-cidadania-marcado-automatico-de</t>
+          <t>BR-plan-plurianual-de-la-ciudad-de-natal</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -24538,12 +24538,12 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Portal e-Cidadania: Marcado automático de respuestas ciudadanas en videos de audiencias públicas</t>
+          <t>Plan Plurianual de la ciudad de Natal</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Plataforma activa; posible nivel 3 si se verifica recurrencia (override)</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -24565,51 +24565,51 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>CL-cabildos-2016</t>
+          <t>BR-portal-e-cidadania-marcado-automatico-de</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Cabildos 2016</t>
+          <t>Portal e-Cidadania: Marcado automático de respuestas ciudadanas en videos de audiencias públicas</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>recodificación 2026: Plataforma activa; posible nivel 3 si se verifica recurrencia (override)</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>CL-cabildos-2016</t>
+          <t>BR-portal-e-cidadania-marcado-automatico-de</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>Cabildos 2016</t>
+          <t>Portal e-Cidadania: Marcado automático de respuestas ciudadanas en videos de audiencias públicas</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: BCN: otra institución pública vs gobierno nacional</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -24631,14 +24631,14 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>CL-estrategia-de-gobierno-digital-informe-p</t>
+          <t>CL-cabildos-2016</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -24648,19 +24648,19 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>Estrategia de Gobierno Digital. Informe proceso participativo segunda consulta ciudadana</t>
+          <t>Cabildos 2016</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>recodificación 2026: BCN: otra institución pública vs gobierno nacional</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>CL-estrategia-de-gobierno-digital-informe-p</t>
+          <t>CL-cabildos-2016</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -24670,7 +24670,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Estrategia de Gobierno Digital. Informe proceso participativo segunda consulta ciudadana</t>
+          <t>Cabildos 2016</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -24682,7 +24682,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>CL-estudio-dialogos-percepciones-de-futuro</t>
+          <t>CL-estrategia-de-gobierno-digital-informe-p</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -24692,7 +24692,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Estudio dIAlogos - Percepciones de Futuro</t>
+          <t>Estrategia de Gobierno Digital. Informe proceso participativo segunda consulta ciudadana</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -24704,7 +24704,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>CL-estudio-dialogos-percepciones-de-futuro</t>
+          <t>CL-estrategia-de-gobierno-digital-informe-p</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -24714,7 +24714,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Estudio dIAlogos - Percepciones de Futuro</t>
+          <t>Estrategia de Gobierno Digital. Informe proceso participativo segunda consulta ciudadana</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -24726,7 +24726,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>CL-jornada-de-escucha-lanzamiento-instituto</t>
+          <t>CL-estudio-dialogos-percepciones-de-futuro</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -24736,7 +24736,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Jornada de Escucha Lanzamiento Instituto de Políticas Públicas UNAB</t>
+          <t>Estudio dIAlogos - Percepciones de Futuro</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -24748,7 +24748,7 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>CL-jornada-de-escucha-lanzamiento-instituto</t>
+          <t>CL-estudio-dialogos-percepciones-de-futuro</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -24758,7 +24758,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Jornada de Escucha Lanzamiento Instituto de Políticas Públicas UNAB</t>
+          <t>Estudio dIAlogos - Percepciones de Futuro</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -24770,7 +24770,7 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>CL-la-voz-de-los-nuevos-votantes</t>
+          <t>CL-jornada-de-escucha-lanzamiento-instituto</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -24780,7 +24780,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>La voz de los nuevos votantes</t>
+          <t>Jornada de Escucha Lanzamiento Instituto de Políticas Públicas UNAB</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -24792,7 +24792,7 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>CL-la-voz-de-los-nuevos-votantes</t>
+          <t>CL-jornada-de-escucha-lanzamiento-instituto</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -24802,7 +24802,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>La voz de los nuevos votantes</t>
+          <t>Jornada de Escucha Lanzamiento Instituto de Políticas Públicas UNAB</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -24814,7 +24814,7 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>CL-participacion-ciudadana-proceso-constitu-2</t>
+          <t>CL-la-voz-de-los-nuevos-votantes</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -24824,7 +24824,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Participación Ciudadana Proceso Constitucional</t>
+          <t>La voz de los nuevos votantes</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -24836,7 +24836,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>CL-participacion-ciudadana-proceso-constitu-2</t>
+          <t>CL-la-voz-de-los-nuevos-votantes</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -24846,12 +24846,12 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Participación Ciudadana Proceso Constitucional</t>
+          <t>La voz de los nuevos votantes</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Aplica a los dos casos homónimos (autoconvocados y audiencias)</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -24873,14 +24873,14 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>CL-participacion-ciudadana-proceso-constitu</t>
+          <t>CL-participacion-ciudadana-proceso-constitu-2</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -24895,14 +24895,14 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>recodificación 2026: Aplica a los dos casos homónimos (autoconvocados y audiencias)</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>CL-participacion-ciudadana-proceso-constitu</t>
+          <t>CL-participacion-ciudadana-proceso-constitu-2</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -24917,7 +24917,7 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Aplica a los dos casos homónimos (autoconvocados y audiencias)</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -24939,14 +24939,14 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>CL-tenemos-que-hablar-de-chile</t>
+          <t>CL-participacion-ciudadana-proceso-constitu</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -24956,19 +24956,19 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Tenemos que hablar de Chile</t>
+          <t>Participación Ciudadana Proceso Constitucional</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>recodificación 2026: Aplica a los dos casos homónimos (autoconvocados y audiencias)</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>CL-tenemos-que-hablar-de-chile</t>
+          <t>CL-participacion-ciudadana-proceso-constitu</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -24978,12 +24978,12 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Tenemos que hablar de Chile</t>
+          <t>Participación Ciudadana Proceso Constitucional</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Escenario B: caso en revisión (puede salir)</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -25005,14 +25005,14 @@
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>CL-un-encuentro-para-la-equidad-de-genero-e</t>
+          <t>CL-tenemos-que-hablar-de-chile</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -25022,19 +25022,19 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Un encuentro para la equidad de género en la movilidad en Chile</t>
+          <t>Tenemos que hablar de Chile</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>recodificación 2026: Escenario B: caso en revisión (puede salir)</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>CL-un-encuentro-para-la-equidad-de-genero-e</t>
+          <t>CL-tenemos-que-hablar-de-chile</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -25044,7 +25044,7 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Un encuentro para la equidad de género en la movilidad en Chile</t>
+          <t>Tenemos que hablar de Chile</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -25056,39 +25056,39 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>CO-chatico</t>
+          <t>CL-un-encuentro-para-la-equidad-de-genero-e</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Chatico</t>
+          <t>Un encuentro para la equidad de género en la movilidad en Chile</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>CO-chatico</t>
+          <t>CL-un-encuentro-para-la-equidad-de-genero-e</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Chatico</t>
+          <t>Un encuentro para la equidad de género en la movilidad en Chile</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -25100,7 +25100,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>CO-descongestion-de-solicitudes-diarias-del</t>
+          <t>CO-chatico</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -25110,19 +25110,19 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Descongestión de solicitudes diarias del programa Ingreso Solidario</t>
+          <t>Chatico</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>CO-descongestion-de-solicitudes-diarias-del</t>
+          <t>CO-chatico</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
@@ -25132,12 +25132,12 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>Descongestión de solicitudes diarias del programa Ingreso Solidario</t>
+          <t>Chatico</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Exclusión FIRME (recodificación 2026): atención/apoyo, no contenido participativo</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -25159,14 +25159,14 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>CO-echo-hablamed-medellin</t>
+          <t>CO-descongestion-de-solicitudes-diarias-del</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
@@ -25176,19 +25176,19 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>ECHO – HáblameD Medellín</t>
+          <t>Descongestión de solicitudes diarias del programa Ingreso Solidario</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
+          <t>recodificación 2026: Exclusión FIRME (recodificación 2026): atención/apoyo, no contenido participativo</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>CO-echo-hablamed-medellin</t>
+          <t>CO-descongestion-de-solicitudes-diarias-del</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -25198,7 +25198,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>ECHO – HáblameD Medellín</t>
+          <t>Descongestión de solicitudes diarias del programa Ingreso Solidario</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -25210,7 +25210,7 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>CO-tenemos-que-hablar-de-colombia</t>
+          <t>CO-echo-hablamed-medellin</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
@@ -25220,19 +25220,19 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Tenemos que hablar de Colombia</t>
+          <t>ECHO – HáblameD Medellín</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>CO-tenemos-que-hablar-de-colombia</t>
+          <t>CO-echo-hablamed-medellin</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -25242,7 +25242,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Tenemos que hablar de Colombia</t>
+          <t>ECHO – HáblameD Medellín</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -25254,17 +25254,17 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>CR-u-report-costa-rica-chatbot-juvenil</t>
+          <t>CO-tenemos-que-hablar-de-colombia</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>U-Report Costa Rica – chatbot juvenil</t>
+          <t>Tenemos que hablar de Colombia</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -25276,17 +25276,17 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>CR-u-report-costa-rica-chatbot-juvenil</t>
+          <t>CO-tenemos-que-hablar-de-colombia</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>U-Report Costa Rica – chatbot juvenil</t>
+          <t>Tenemos que hablar de Colombia</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -25298,7 +25298,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>CR-diara</t>
+          <t>CR-u-report-costa-rica-chatbot-juvenil</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -25308,7 +25308,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>dIAra</t>
+          <t>U-Report Costa Rica – chatbot juvenil</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -25320,7 +25320,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>CR-diara</t>
+          <t>CR-u-report-costa-rica-chatbot-juvenil</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -25330,12 +25330,12 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>dIAra</t>
+          <t>U-Report Costa Rica – chatbot juvenil</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Revisar rol_IA: monitoreo de obras (traducción política)</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -25357,51 +25357,51 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>DO-ciudadania</t>
+          <t>CR-diara</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>CiudadanIA</t>
+          <t>dIAra</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
+          <t>recodificación 2026: Revisar rol_IA: monitoreo de obras (traducción política)</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>DO-ciudadania</t>
+          <t>CR-diara</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>CiudadanIA</t>
+          <t>dIAra</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Escenario B: caso en revisión (puede salir). GENIA: empresa/soc. civil (ambiguo)</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -25423,46 +25423,46 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>EC-paga-ia</t>
+          <t>DO-ciudadania</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAGA IA </t>
+          <t>CiudadanIA</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
+          <t>recodificación 2026: Escenario B: caso en revisión (puede salir). GENIA: empresa/soc. civil (ambiguo)</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>EC-paga-ia</t>
+          <t>DO-ciudadania</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAGA IA </t>
+          <t>CiudadanIA</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -25474,39 +25474,39 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>GT-guatemala-joven-conversa</t>
+          <t>EC-paga-ia</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guatemala Joven Conversa </t>
+          <t xml:space="preserve">PAGA IA </t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>usa_LLM_generativa derivado de Tipos de IA (BBDD 2025: contiene 'LLM')</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>GT-guatemala-joven-conversa</t>
+          <t>EC-paga-ia</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guatemala Joven Conversa </t>
+          <t xml:space="preserve">PAGA IA </t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -25518,17 +25518,17 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>HN-redpublica-iverify</t>
+          <t>GT-guatemala-joven-conversa</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>HN</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedPública + iVerify </t>
+          <t xml:space="preserve">Guatemala Joven Conversa </t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -25540,17 +25540,17 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>HN-redpublica-iverify</t>
+          <t>GT-guatemala-joven-conversa</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>HN</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">RedPública + iVerify </t>
+          <t xml:space="preserve">Guatemala Joven Conversa </t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -25562,17 +25562,17 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>MX-presupuesto-creces</t>
+          <t>HN-redpublica-iverify</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>HN</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto CRECES</t>
+          <t xml:space="preserve">RedPública + iVerify </t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -25584,17 +25584,17 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>MX-presupuesto-creces</t>
+          <t>HN-redpublica-iverify</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>HN</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto CRECES</t>
+          <t xml:space="preserve">RedPública + iVerify </t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -25606,7 +25606,7 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>MX-sufragio-seguro</t>
+          <t>MX-presupuesto-creces</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -25616,7 +25616,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>Sufragio seguro</t>
+          <t>Presupuesto CRECES</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -25628,7 +25628,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>MX-sufragio-seguro</t>
+          <t>MX-presupuesto-creces</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -25638,12 +25638,12 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Sufragio seguro</t>
+          <t>Presupuesto CRECES</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Exclusión FIRME (recodificación 2026): integridad/proceso electoral, no contenido</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -25665,51 +25665,51 @@
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>PE-consulta-ciudadana-sobre-el-proyecto-nac</t>
+          <t>MX-sufragio-seguro</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
+          <t>Sufragio seguro</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>recodificación 2026: Exclusión FIRME (recodificación 2026): integridad/proceso electoral, no contenido</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>PE-consulta-ciudadana-sobre-el-proyecto-nac</t>
+          <t>MX-sufragio-seguro</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
+          <t>Sufragio seguro</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: CNE: organismo autónomo (otra pública) vs gobierno nacional</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -25731,14 +25731,14 @@
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>PE-sistema-de-computo-con-ia-para-las-elecc</t>
+          <t>PE-consulta-ciudadana-sobre-el-proyecto-nac</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -25748,19 +25748,19 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Sistema de cómputo con IA para las Elecciones Generales 2026</t>
+          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+          <t>recodificación 2026: CNE: organismo autónomo (otra pública) vs gobierno nacional</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>PE-sistema-de-computo-con-ia-para-las-elecc</t>
+          <t>PE-consulta-ciudadana-sobre-el-proyecto-nac</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -25770,12 +25770,12 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Sistema de cómputo con IA para las Elecciones Generales 2026</t>
+          <t>Consulta Ciudadana sobre el Proyecto Nacional de Educación</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>recodificación 2026: Exclusión FIRME (recodificación 2026): conteo electoral (OCR), no participación; estado 'Próximamente' = anuncio</t>
+          <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
@@ -25797,12 +25797,56 @@
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
+          <t>usa_LLM_generativa='no' derivado de Tipos de IA 2025 (sin 'LLM'); verificar si cambió en 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>PE-sistema-de-computo-con-ia-para-las-elecc</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>Sistema de cómputo con IA para las Elecciones Generales 2026</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>recodificación 2026: Exclusión FIRME (recodificación 2026): conteo electoral (OCR), no participación; estado 'Próximamente' = anuncio</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>PE-sistema-de-computo-con-ia-para-las-elecc</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>Sistema de cómputo con IA para las Elecciones Generales 2026</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
           <t>Datos brutos del índice ILIA 2025 (BBDD validada por el equipo); recodificación 2026 (convocante 7-cat, nivel 0-3) y reverificación de actividad 2026.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D197"/>
+  <autoFilter ref="A1:D199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>